<commit_message>
Fix IRI unit_sales/dollar_sales scaling to eliminate cross-source volume warning
IRI unit_sales was stored at IRI_MULT (5.5×) scale while POS is at retailer
scale, causing an 82% cross-source mismatch warning on every fixture. Store
both at retailer scale — market_share_* columns are pre-computed correctly
(IRI_MULT cancels in the ratio) and avg_net_price is stored directly as price,
so nothing else is affected. Zero validation warnings on all three fixtures.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stella/test_fixtures/inventory_risk/iri_data.xlsx
+++ b/stella/test_fixtures/inventory_risk/iri_data.xlsx
@@ -499,10 +499,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>16648.35</v>
+        <v>3026.97</v>
       </c>
       <c r="E2" t="n">
-        <v>2646.8</v>
+        <v>481.2</v>
       </c>
       <c r="F2" t="n">
         <v>6.29</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>17154.19</v>
+        <v>3118.94</v>
       </c>
       <c r="E3" t="n">
-        <v>2727.2</v>
+        <v>495.9</v>
       </c>
       <c r="F3" t="n">
         <v>6.29</v>
@@ -571,10 +571,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>17913.5</v>
+        <v>3257</v>
       </c>
       <c r="E4" t="n">
-        <v>2847.9</v>
+        <v>517.8</v>
       </c>
       <c r="F4" t="n">
         <v>6.29</v>
@@ -607,10 +607,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15485.62</v>
+        <v>2815.57</v>
       </c>
       <c r="E5" t="n">
-        <v>2386.1</v>
+        <v>433.8</v>
       </c>
       <c r="F5" t="n">
         <v>6.49</v>
@@ -643,10 +643,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16383.63</v>
+        <v>2978.84</v>
       </c>
       <c r="E6" t="n">
-        <v>2524.4</v>
+        <v>459</v>
       </c>
       <c r="F6" t="n">
         <v>6.49</v>
@@ -679,10 +679,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15751.28</v>
+        <v>2863.87</v>
       </c>
       <c r="E7" t="n">
-        <v>2427</v>
+        <v>441.3</v>
       </c>
       <c r="F7" t="n">
         <v>6.49</v>
@@ -715,10 +715,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>17000.91</v>
+        <v>3091.07</v>
       </c>
       <c r="E8" t="n">
-        <v>3962.9</v>
+        <v>720.5</v>
       </c>
       <c r="F8" t="n">
         <v>4.29</v>
@@ -751,10 +751,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16841.63</v>
+        <v>3062.12</v>
       </c>
       <c r="E9" t="n">
-        <v>3925.8</v>
+        <v>713.8</v>
       </c>
       <c r="F9" t="n">
         <v>4.29</v>
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17026.14</v>
+        <v>3095.66</v>
       </c>
       <c r="E10" t="n">
-        <v>3968.8</v>
+        <v>721.6</v>
       </c>
       <c r="F10" t="n">
         <v>4.29</v>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>14289.46</v>
+        <v>2598.08</v>
       </c>
       <c r="E11" t="n">
-        <v>3493.8</v>
+        <v>635.2</v>
       </c>
       <c r="F11" t="n">
         <v>4.09</v>
@@ -859,10 +859,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>14658.35</v>
+        <v>2665.16</v>
       </c>
       <c r="E12" t="n">
-        <v>3583.9</v>
+        <v>651.6</v>
       </c>
       <c r="F12" t="n">
         <v>4.09</v>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>14948.42</v>
+        <v>2717.9</v>
       </c>
       <c r="E13" t="n">
-        <v>3654.9</v>
+        <v>664.5</v>
       </c>
       <c r="F13" t="n">
         <v>4.09</v>
@@ -931,10 +931,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>12026.26</v>
+        <v>2186.59</v>
       </c>
       <c r="E14" t="n">
-        <v>4310.5</v>
+        <v>783.7</v>
       </c>
       <c r="F14" t="n">
         <v>2.79</v>
@@ -967,10 +967,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>12011.57</v>
+        <v>2183.92</v>
       </c>
       <c r="E15" t="n">
-        <v>4305.2</v>
+        <v>782.8</v>
       </c>
       <c r="F15" t="n">
         <v>2.79</v>
@@ -1003,10 +1003,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11811.66</v>
+        <v>2147.57</v>
       </c>
       <c r="E16" t="n">
-        <v>4233.6</v>
+        <v>769.7</v>
       </c>
       <c r="F16" t="n">
         <v>2.79</v>
@@ -1039,10 +1039,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>17855.02</v>
+        <v>3246.37</v>
       </c>
       <c r="E17" t="n">
-        <v>2838.6</v>
+        <v>516.1</v>
       </c>
       <c r="F17" t="n">
         <v>6.29</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>17881.32</v>
+        <v>3251.15</v>
       </c>
       <c r="E18" t="n">
-        <v>2842.8</v>
+        <v>516.9</v>
       </c>
       <c r="F18" t="n">
         <v>6.29</v>
@@ -1111,10 +1111,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>17065.25</v>
+        <v>3102.77</v>
       </c>
       <c r="E19" t="n">
-        <v>2713.1</v>
+        <v>493.3</v>
       </c>
       <c r="F19" t="n">
         <v>6.29</v>
@@ -1147,10 +1147,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>15637.58</v>
+        <v>2843.2</v>
       </c>
       <c r="E20" t="n">
-        <v>2409.5</v>
+        <v>438.1</v>
       </c>
       <c r="F20" t="n">
         <v>6.49</v>
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>15692.37</v>
+        <v>2853.16</v>
       </c>
       <c r="E21" t="n">
-        <v>2417.9</v>
+        <v>439.6</v>
       </c>
       <c r="F21" t="n">
         <v>6.49</v>
@@ -1219,10 +1219,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>15535.89</v>
+        <v>2824.71</v>
       </c>
       <c r="E22" t="n">
-        <v>2393.8</v>
+        <v>435.2</v>
       </c>
       <c r="F22" t="n">
         <v>6.49</v>
@@ -1255,10 +1255,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>16014.54</v>
+        <v>2911.74</v>
       </c>
       <c r="E23" t="n">
-        <v>3733</v>
+        <v>678.7</v>
       </c>
       <c r="F23" t="n">
         <v>4.29</v>
@@ -1291,10 +1291,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>15950.06</v>
+        <v>2900.01</v>
       </c>
       <c r="E24" t="n">
-        <v>3718</v>
+        <v>676</v>
       </c>
       <c r="F24" t="n">
         <v>4.29</v>
@@ -1327,10 +1327,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>17163.71</v>
+        <v>3120.68</v>
       </c>
       <c r="E25" t="n">
-        <v>4000.9</v>
+        <v>727.4</v>
       </c>
       <c r="F25" t="n">
         <v>4.29</v>
@@ -1363,10 +1363,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>14123.51</v>
+        <v>2567.91</v>
       </c>
       <c r="E26" t="n">
-        <v>3453.2</v>
+        <v>627.9</v>
       </c>
       <c r="F26" t="n">
         <v>4.09</v>
@@ -1399,10 +1399,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>14191.92</v>
+        <v>2580.35</v>
       </c>
       <c r="E27" t="n">
-        <v>3469.9</v>
+        <v>630.9</v>
       </c>
       <c r="F27" t="n">
         <v>4.09</v>
@@ -1435,10 +1435,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>15004.55</v>
+        <v>2728.1</v>
       </c>
       <c r="E28" t="n">
-        <v>3668.6</v>
+        <v>667</v>
       </c>
       <c r="F28" t="n">
         <v>4.09</v>
@@ -1471,10 +1471,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>12354.8</v>
+        <v>2246.33</v>
       </c>
       <c r="E29" t="n">
-        <v>4428.2</v>
+        <v>805.1</v>
       </c>
       <c r="F29" t="n">
         <v>2.79</v>
@@ -1507,10 +1507,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>12545.5</v>
+        <v>2281</v>
       </c>
       <c r="E30" t="n">
-        <v>4496.6</v>
+        <v>817.6</v>
       </c>
       <c r="F30" t="n">
         <v>2.79</v>
@@ -1543,10 +1543,10 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>12404.57</v>
+        <v>2255.38</v>
       </c>
       <c r="E31" t="n">
-        <v>4446.1</v>
+        <v>808.4</v>
       </c>
       <c r="F31" t="n">
         <v>2.79</v>
@@ -1579,10 +1579,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>17790.7</v>
+        <v>3234.67</v>
       </c>
       <c r="E32" t="n">
-        <v>2828.4</v>
+        <v>514.3</v>
       </c>
       <c r="F32" t="n">
         <v>6.29</v>
@@ -1615,10 +1615,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>16713.18</v>
+        <v>3038.76</v>
       </c>
       <c r="E33" t="n">
-        <v>2657.1</v>
+        <v>483.1</v>
       </c>
       <c r="F33" t="n">
         <v>6.29</v>
@@ -1651,10 +1651,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>17664.24</v>
+        <v>3211.68</v>
       </c>
       <c r="E34" t="n">
-        <v>2808.3</v>
+        <v>510.6</v>
       </c>
       <c r="F34" t="n">
         <v>6.29</v>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>15815.6</v>
+        <v>2875.56</v>
       </c>
       <c r="E35" t="n">
-        <v>2436.9</v>
+        <v>443.1</v>
       </c>
       <c r="F35" t="n">
         <v>6.49</v>
@@ -1723,10 +1723,10 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>15698.6</v>
+        <v>2854.29</v>
       </c>
       <c r="E36" t="n">
-        <v>2418.9</v>
+        <v>439.8</v>
       </c>
       <c r="F36" t="n">
         <v>6.49</v>
@@ -1759,10 +1759,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>16305.49</v>
+        <v>2964.63</v>
       </c>
       <c r="E37" t="n">
-        <v>2512.4</v>
+        <v>456.8</v>
       </c>
       <c r="F37" t="n">
         <v>6.49</v>
@@ -1795,10 +1795,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>17057.97</v>
+        <v>3101.45</v>
       </c>
       <c r="E38" t="n">
-        <v>3976.2</v>
+        <v>722.9</v>
       </c>
       <c r="F38" t="n">
         <v>4.29</v>
@@ -1831,10 +1831,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>16245.65</v>
+        <v>2953.76</v>
       </c>
       <c r="E39" t="n">
-        <v>3786.9</v>
+        <v>688.5</v>
       </c>
       <c r="F39" t="n">
         <v>4.29</v>
@@ -1867,10 +1867,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>16607.45</v>
+        <v>3019.54</v>
       </c>
       <c r="E40" t="n">
-        <v>3871.2</v>
+        <v>703.9</v>
       </c>
       <c r="F40" t="n">
         <v>4.29</v>
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>14375.91</v>
+        <v>2613.8</v>
       </c>
       <c r="E41" t="n">
-        <v>3514.9</v>
+        <v>639.1</v>
       </c>
       <c r="F41" t="n">
         <v>4.09</v>
@@ -1939,10 +1939,10 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>14685.25</v>
+        <v>2670.05</v>
       </c>
       <c r="E42" t="n">
-        <v>3590.5</v>
+        <v>652.8</v>
       </c>
       <c r="F42" t="n">
         <v>4.09</v>
@@ -1975,10 +1975,10 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>14764.3</v>
+        <v>2684.42</v>
       </c>
       <c r="E43" t="n">
-        <v>3609.9</v>
+        <v>656.3</v>
       </c>
       <c r="F43" t="n">
         <v>4.09</v>
@@ -2011,10 +2011,10 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>12384.36</v>
+        <v>2251.7</v>
       </c>
       <c r="E44" t="n">
-        <v>4438.8</v>
+        <v>807.1</v>
       </c>
       <c r="F44" t="n">
         <v>2.79</v>
@@ -2047,10 +2047,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>12397.33</v>
+        <v>2254.06</v>
       </c>
       <c r="E45" t="n">
-        <v>4443.5</v>
+        <v>807.9</v>
       </c>
       <c r="F45" t="n">
         <v>2.79</v>
@@ -2083,10 +2083,10 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>11917.62</v>
+        <v>2166.84</v>
       </c>
       <c r="E46" t="n">
-        <v>4271.5</v>
+        <v>776.6</v>
       </c>
       <c r="F46" t="n">
         <v>2.79</v>
@@ -2119,10 +2119,10 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>17296.38</v>
+        <v>3144.8</v>
       </c>
       <c r="E47" t="n">
-        <v>2749.8</v>
+        <v>500</v>
       </c>
       <c r="F47" t="n">
         <v>6.29</v>
@@ -2155,10 +2155,10 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>17463.17</v>
+        <v>3175.12</v>
       </c>
       <c r="E48" t="n">
-        <v>2776.3</v>
+        <v>504.8</v>
       </c>
       <c r="F48" t="n">
         <v>6.29</v>
@@ -2191,10 +2191,10 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>17889.73</v>
+        <v>3252.68</v>
       </c>
       <c r="E49" t="n">
-        <v>2844.2</v>
+        <v>517.1</v>
       </c>
       <c r="F49" t="n">
         <v>6.29</v>
@@ -2227,10 +2227,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>16052.23</v>
+        <v>2918.59</v>
       </c>
       <c r="E50" t="n">
-        <v>2473.4</v>
+        <v>449.7</v>
       </c>
       <c r="F50" t="n">
         <v>6.49</v>
@@ -2263,10 +2263,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>16099.58</v>
+        <v>2927.2</v>
       </c>
       <c r="E51" t="n">
-        <v>2480.7</v>
+        <v>451</v>
       </c>
       <c r="F51" t="n">
         <v>6.49</v>
@@ -2299,10 +2299,10 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>16193.82</v>
+        <v>2944.33</v>
       </c>
       <c r="E52" t="n">
-        <v>2495.2</v>
+        <v>453.7</v>
       </c>
       <c r="F52" t="n">
         <v>6.49</v>
@@ -2335,10 +2335,10 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>16830.33</v>
+        <v>3060.06</v>
       </c>
       <c r="E53" t="n">
-        <v>3923.2</v>
+        <v>713.3</v>
       </c>
       <c r="F53" t="n">
         <v>4.29</v>
@@ -2371,10 +2371,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>15950.78</v>
+        <v>2900.14</v>
       </c>
       <c r="E54" t="n">
-        <v>3718.1</v>
+        <v>676</v>
       </c>
       <c r="F54" t="n">
         <v>4.29</v>
@@ -2407,10 +2407,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>16537.23</v>
+        <v>3006.77</v>
       </c>
       <c r="E55" t="n">
-        <v>3854.8</v>
+        <v>700.9</v>
       </c>
       <c r="F55" t="n">
         <v>4.29</v>
@@ -2443,10 +2443,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>14600.22</v>
+        <v>2654.58</v>
       </c>
       <c r="E56" t="n">
-        <v>3569.7</v>
+        <v>649</v>
       </c>
       <c r="F56" t="n">
         <v>4.09</v>
@@ -2479,10 +2479,10 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>15115.01</v>
+        <v>2748.18</v>
       </c>
       <c r="E57" t="n">
-        <v>3695.6</v>
+        <v>671.9</v>
       </c>
       <c r="F57" t="n">
         <v>4.09</v>
@@ -2515,10 +2515,10 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>14614.15</v>
+        <v>2657.12</v>
       </c>
       <c r="E58" t="n">
-        <v>3573.1</v>
+        <v>649.7</v>
       </c>
       <c r="F58" t="n">
         <v>4.09</v>
@@ -2551,10 +2551,10 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>12244.89</v>
+        <v>2226.34</v>
       </c>
       <c r="E59" t="n">
-        <v>4388.8</v>
+        <v>798</v>
       </c>
       <c r="F59" t="n">
         <v>2.79</v>
@@ -2587,10 +2587,10 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>12729.92</v>
+        <v>2314.53</v>
       </c>
       <c r="E60" t="n">
-        <v>4562.7</v>
+        <v>829.6</v>
       </c>
       <c r="F60" t="n">
         <v>2.79</v>
@@ -2623,10 +2623,10 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>12227.46</v>
+        <v>2223.17</v>
       </c>
       <c r="E61" t="n">
-        <v>4382.6</v>
+        <v>796.8</v>
       </c>
       <c r="F61" t="n">
         <v>2.79</v>
@@ -2659,10 +2659,10 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>27525.42</v>
+        <v>5004.62</v>
       </c>
       <c r="E62" t="n">
-        <v>5461.4</v>
+        <v>993</v>
       </c>
       <c r="F62" t="n">
         <v>5.04</v>
@@ -2695,10 +2695,10 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>28295.78</v>
+        <v>5144.69</v>
       </c>
       <c r="E63" t="n">
-        <v>5614.2</v>
+        <v>1020.8</v>
       </c>
       <c r="F63" t="n">
         <v>5.04</v>
@@ -2731,10 +2731,10 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>27122.75</v>
+        <v>4931.41</v>
       </c>
       <c r="E64" t="n">
-        <v>5381.5</v>
+        <v>978.5</v>
       </c>
       <c r="F64" t="n">
         <v>5.04</v>
@@ -2767,10 +2767,10 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14925.78</v>
+        <v>2713.78</v>
       </c>
       <c r="E65" t="n">
-        <v>2299.8</v>
+        <v>418.1</v>
       </c>
       <c r="F65" t="n">
         <v>6.49</v>
@@ -2803,10 +2803,10 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>14456.72</v>
+        <v>2628.49</v>
       </c>
       <c r="E66" t="n">
-        <v>2227.5</v>
+        <v>405</v>
       </c>
       <c r="F66" t="n">
         <v>6.49</v>
@@ -2839,10 +2839,10 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>14752.65</v>
+        <v>2682.3</v>
       </c>
       <c r="E67" t="n">
-        <v>2273.1</v>
+        <v>413.3</v>
       </c>
       <c r="F67" t="n">
         <v>6.49</v>
@@ -2875,10 +2875,10 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>16299.46</v>
+        <v>2963.54</v>
       </c>
       <c r="E68" t="n">
-        <v>3799.4</v>
+        <v>690.8</v>
       </c>
       <c r="F68" t="n">
         <v>4.29</v>
@@ -2911,10 +2911,10 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>16488.59</v>
+        <v>2997.93</v>
       </c>
       <c r="E69" t="n">
-        <v>3843.5</v>
+        <v>698.8</v>
       </c>
       <c r="F69" t="n">
         <v>4.29</v>
@@ -2947,10 +2947,10 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>15505.67</v>
+        <v>2819.21</v>
       </c>
       <c r="E70" t="n">
-        <v>3614.4</v>
+        <v>657.2</v>
       </c>
       <c r="F70" t="n">
         <v>4.29</v>
@@ -2983,10 +2983,10 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>13941.3</v>
+        <v>2534.78</v>
       </c>
       <c r="E71" t="n">
-        <v>3408.6</v>
+        <v>619.8</v>
       </c>
       <c r="F71" t="n">
         <v>4.09</v>
@@ -3019,10 +3019,10 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>13899.93</v>
+        <v>2527.26</v>
       </c>
       <c r="E72" t="n">
-        <v>3398.5</v>
+        <v>617.9</v>
       </c>
       <c r="F72" t="n">
         <v>4.09</v>
@@ -3055,10 +3055,10 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>13914.04</v>
+        <v>2529.83</v>
       </c>
       <c r="E73" t="n">
-        <v>3402</v>
+        <v>618.5</v>
       </c>
       <c r="F73" t="n">
         <v>4.09</v>
@@ -3091,10 +3091,10 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>12233.4</v>
+        <v>2224.25</v>
       </c>
       <c r="E74" t="n">
-        <v>4384.7</v>
+        <v>797.2</v>
       </c>
       <c r="F74" t="n">
         <v>2.79</v>
@@ -3127,10 +3127,10 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>12633.07</v>
+        <v>2296.92</v>
       </c>
       <c r="E75" t="n">
-        <v>4528</v>
+        <v>823.3</v>
       </c>
       <c r="F75" t="n">
         <v>2.79</v>
@@ -3163,10 +3163,10 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>12629.92</v>
+        <v>2296.35</v>
       </c>
       <c r="E76" t="n">
-        <v>4526.9</v>
+        <v>823.1</v>
       </c>
       <c r="F76" t="n">
         <v>2.79</v>
@@ -3199,10 +3199,10 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>27824.85</v>
+        <v>5059.06</v>
       </c>
       <c r="E77" t="n">
-        <v>5520.8</v>
+        <v>1003.8</v>
       </c>
       <c r="F77" t="n">
         <v>5.04</v>
@@ -3235,10 +3235,10 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>27854.78</v>
+        <v>5064.51</v>
       </c>
       <c r="E78" t="n">
-        <v>5526.7</v>
+        <v>1004.9</v>
       </c>
       <c r="F78" t="n">
         <v>5.04</v>
@@ -3271,10 +3271,10 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>27732.2</v>
+        <v>5042.22</v>
       </c>
       <c r="E79" t="n">
-        <v>5502.4</v>
+        <v>1000.4</v>
       </c>
       <c r="F79" t="n">
         <v>5.04</v>
@@ -3307,10 +3307,10 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>14614.54</v>
+        <v>2657.19</v>
       </c>
       <c r="E80" t="n">
-        <v>2251.9</v>
+        <v>409.4</v>
       </c>
       <c r="F80" t="n">
         <v>6.49</v>
@@ -3343,10 +3343,10 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>14350.45</v>
+        <v>2609.17</v>
       </c>
       <c r="E81" t="n">
-        <v>2211.2</v>
+        <v>402</v>
       </c>
       <c r="F81" t="n">
         <v>6.49</v>
@@ -3379,10 +3379,10 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>14744.65</v>
+        <v>2680.85</v>
       </c>
       <c r="E82" t="n">
-        <v>2271.9</v>
+        <v>413.1</v>
       </c>
       <c r="F82" t="n">
         <v>6.49</v>
@@ -3415,10 +3415,10 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>15644.7</v>
+        <v>2844.49</v>
       </c>
       <c r="E83" t="n">
-        <v>3646.8</v>
+        <v>663.1</v>
       </c>
       <c r="F83" t="n">
         <v>4.29</v>
@@ -3451,10 +3451,10 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>15641.06</v>
+        <v>2843.83</v>
       </c>
       <c r="E84" t="n">
-        <v>3645.9</v>
+        <v>662.9</v>
       </c>
       <c r="F84" t="n">
         <v>4.29</v>
@@ -3487,10 +3487,10 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>15382.99</v>
+        <v>2796.91</v>
       </c>
       <c r="E85" t="n">
-        <v>3585.8</v>
+        <v>652</v>
       </c>
       <c r="F85" t="n">
         <v>4.29</v>
@@ -3523,10 +3523,10 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>13829.9</v>
+        <v>2514.53</v>
       </c>
       <c r="E86" t="n">
-        <v>3381.4</v>
+        <v>614.8</v>
       </c>
       <c r="F86" t="n">
         <v>4.09</v>
@@ -3559,10 +3559,10 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>14580.82</v>
+        <v>2651.06</v>
       </c>
       <c r="E87" t="n">
-        <v>3565</v>
+        <v>648.2</v>
       </c>
       <c r="F87" t="n">
         <v>4.09</v>
@@ -3595,10 +3595,10 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>14122.15</v>
+        <v>2567.66</v>
       </c>
       <c r="E88" t="n">
-        <v>3452.8</v>
+        <v>627.8</v>
       </c>
       <c r="F88" t="n">
         <v>4.09</v>
@@ -3631,10 +3631,10 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>11888.66</v>
+        <v>2161.57</v>
       </c>
       <c r="E89" t="n">
-        <v>4261.2</v>
+        <v>774.8</v>
       </c>
       <c r="F89" t="n">
         <v>2.79</v>
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>12405.39</v>
+        <v>2255.52</v>
       </c>
       <c r="E90" t="n">
-        <v>4446.4</v>
+        <v>808.4</v>
       </c>
       <c r="F90" t="n">
         <v>2.79</v>
@@ -3703,10 +3703,10 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12205.72</v>
+        <v>2219.22</v>
       </c>
       <c r="E91" t="n">
-        <v>4374.8</v>
+        <v>795.4</v>
       </c>
       <c r="F91" t="n">
         <v>2.79</v>
@@ -3739,10 +3739,10 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>28391.38</v>
+        <v>5162.07</v>
       </c>
       <c r="E92" t="n">
-        <v>5633.2</v>
+        <v>1024.2</v>
       </c>
       <c r="F92" t="n">
         <v>5.04</v>
@@ -3775,10 +3775,10 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>28591.63</v>
+        <v>5198.48</v>
       </c>
       <c r="E93" t="n">
-        <v>5672.9</v>
+        <v>1031.4</v>
       </c>
       <c r="F93" t="n">
         <v>5.04</v>
@@ -3811,10 +3811,10 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>26635.63</v>
+        <v>4842.84</v>
       </c>
       <c r="E94" t="n">
-        <v>5284.8</v>
+        <v>960.9</v>
       </c>
       <c r="F94" t="n">
         <v>5.04</v>
@@ -3847,10 +3847,10 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>14084.77</v>
+        <v>2560.87</v>
       </c>
       <c r="E95" t="n">
-        <v>2170.2</v>
+        <v>394.6</v>
       </c>
       <c r="F95" t="n">
         <v>6.49</v>
@@ -3883,10 +3883,10 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>14923.6</v>
+        <v>2713.38</v>
       </c>
       <c r="E96" t="n">
-        <v>2299.5</v>
+        <v>418.1</v>
       </c>
       <c r="F96" t="n">
         <v>6.49</v>
@@ -3919,10 +3919,10 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>14513.72</v>
+        <v>2638.86</v>
       </c>
       <c r="E97" t="n">
-        <v>2236.3</v>
+        <v>406.6</v>
       </c>
       <c r="F97" t="n">
         <v>6.49</v>
@@ -3955,10 +3955,10 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>15411.93</v>
+        <v>2802.17</v>
       </c>
       <c r="E98" t="n">
-        <v>3592.5</v>
+        <v>653.2</v>
       </c>
       <c r="F98" t="n">
         <v>4.29</v>
@@ -3991,10 +3991,10 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15478.84</v>
+        <v>2814.33</v>
       </c>
       <c r="E99" t="n">
-        <v>3608.1</v>
+        <v>656</v>
       </c>
       <c r="F99" t="n">
         <v>4.29</v>
@@ -4027,10 +4027,10 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>16058.78</v>
+        <v>2919.78</v>
       </c>
       <c r="E100" t="n">
-        <v>3743.3</v>
+        <v>680.6</v>
       </c>
       <c r="F100" t="n">
         <v>4.29</v>
@@ -4063,10 +4063,10 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>14438.19</v>
+        <v>2625.12</v>
       </c>
       <c r="E101" t="n">
-        <v>3530.1</v>
+        <v>641.8</v>
       </c>
       <c r="F101" t="n">
         <v>4.09</v>
@@ -4099,10 +4099,10 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>14295.91</v>
+        <v>2599.26</v>
       </c>
       <c r="E102" t="n">
-        <v>3495.3</v>
+        <v>635.5</v>
       </c>
       <c r="F102" t="n">
         <v>4.09</v>
@@ -4135,10 +4135,10 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>14697.26</v>
+        <v>2672.23</v>
       </c>
       <c r="E103" t="n">
-        <v>3593.5</v>
+        <v>653.4</v>
       </c>
       <c r="F103" t="n">
         <v>4.09</v>
@@ -4171,10 +4171,10 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>12147.47</v>
+        <v>2208.63</v>
       </c>
       <c r="E104" t="n">
-        <v>4353.9</v>
+        <v>791.6</v>
       </c>
       <c r="F104" t="n">
         <v>2.79</v>
@@ -4207,10 +4207,10 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>11959.05</v>
+        <v>2174.37</v>
       </c>
       <c r="E105" t="n">
-        <v>4286.4</v>
+        <v>779.3</v>
       </c>
       <c r="F105" t="n">
         <v>2.79</v>
@@ -4243,10 +4243,10 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>12131.1</v>
+        <v>2205.66</v>
       </c>
       <c r="E106" t="n">
-        <v>4348.1</v>
+        <v>790.6</v>
       </c>
       <c r="F106" t="n">
         <v>2.79</v>
@@ -4279,10 +4279,10 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>27155.77</v>
+        <v>4937.41</v>
       </c>
       <c r="E107" t="n">
-        <v>5388</v>
+        <v>979.6</v>
       </c>
       <c r="F107" t="n">
         <v>5.04</v>
@@ -4315,10 +4315,10 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>26705.56</v>
+        <v>4855.56</v>
       </c>
       <c r="E108" t="n">
-        <v>5298.7</v>
+        <v>963.4</v>
       </c>
       <c r="F108" t="n">
         <v>5.04</v>
@@ -4351,10 +4351,10 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>27107.03</v>
+        <v>4928.55</v>
       </c>
       <c r="E109" t="n">
-        <v>5378.4</v>
+        <v>977.9</v>
       </c>
       <c r="F109" t="n">
         <v>5.04</v>
@@ -4387,10 +4387,10 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>14404.31</v>
+        <v>2618.97</v>
       </c>
       <c r="E110" t="n">
-        <v>2219.5</v>
+        <v>403.5</v>
       </c>
       <c r="F110" t="n">
         <v>6.49</v>
@@ -4423,10 +4423,10 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>14356.93</v>
+        <v>2610.35</v>
       </c>
       <c r="E111" t="n">
-        <v>2212.2</v>
+        <v>402.2</v>
       </c>
       <c r="F111" t="n">
         <v>6.49</v>
@@ -4459,10 +4459,10 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>14082.53</v>
+        <v>2560.46</v>
       </c>
       <c r="E112" t="n">
-        <v>2169.9</v>
+        <v>394.5</v>
       </c>
       <c r="F112" t="n">
         <v>6.49</v>
@@ -4495,10 +4495,10 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>16267.35</v>
+        <v>2957.7</v>
       </c>
       <c r="E113" t="n">
-        <v>3791.9</v>
+        <v>689.4</v>
       </c>
       <c r="F113" t="n">
         <v>4.29</v>
@@ -4531,10 +4531,10 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>16395.81</v>
+        <v>2981.06</v>
       </c>
       <c r="E114" t="n">
-        <v>3821.9</v>
+        <v>694.9</v>
       </c>
       <c r="F114" t="n">
         <v>4.29</v>
@@ -4567,10 +4567,10 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>15477.01</v>
+        <v>2814</v>
       </c>
       <c r="E115" t="n">
-        <v>3607.7</v>
+        <v>655.9</v>
       </c>
       <c r="F115" t="n">
         <v>4.29</v>
@@ -4603,10 +4603,10 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>14670.51</v>
+        <v>2667.37</v>
       </c>
       <c r="E116" t="n">
-        <v>3586.9</v>
+        <v>652.2</v>
       </c>
       <c r="F116" t="n">
         <v>4.09</v>
@@ -4639,10 +4639,10 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>13636.04</v>
+        <v>2479.28</v>
       </c>
       <c r="E117" t="n">
-        <v>3334</v>
+        <v>606.2</v>
       </c>
       <c r="F117" t="n">
         <v>4.09</v>
@@ -4675,10 +4675,10 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>14665.28</v>
+        <v>2666.41</v>
       </c>
       <c r="E118" t="n">
-        <v>3585.6</v>
+        <v>651.9</v>
       </c>
       <c r="F118" t="n">
         <v>4.09</v>
@@ -4711,10 +4711,10 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>12592.63</v>
+        <v>2289.57</v>
       </c>
       <c r="E119" t="n">
-        <v>4513.5</v>
+        <v>820.6</v>
       </c>
       <c r="F119" t="n">
         <v>2.79</v>
@@ -4747,10 +4747,10 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>11678.83</v>
+        <v>2123.42</v>
       </c>
       <c r="E120" t="n">
-        <v>4186</v>
+        <v>761.1</v>
       </c>
       <c r="F120" t="n">
         <v>2.79</v>
@@ -4783,10 +4783,10 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>12408.96</v>
+        <v>2256.18</v>
       </c>
       <c r="E121" t="n">
-        <v>4447.7</v>
+        <v>808.7</v>
       </c>
       <c r="F121" t="n">
         <v>2.79</v>
@@ -4819,10 +4819,10 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>13807.52</v>
+        <v>2510.46</v>
       </c>
       <c r="E122" t="n">
-        <v>2195.2</v>
+        <v>399.1</v>
       </c>
       <c r="F122" t="n">
         <v>6.29</v>
@@ -4855,10 +4855,10 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>13848.88</v>
+        <v>2517.98</v>
       </c>
       <c r="E123" t="n">
-        <v>2201.7</v>
+        <v>400.3</v>
       </c>
       <c r="F123" t="n">
         <v>6.29</v>
@@ -4891,10 +4891,10 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>13630.11</v>
+        <v>2478.2</v>
       </c>
       <c r="E124" t="n">
-        <v>2166.9</v>
+        <v>394</v>
       </c>
       <c r="F124" t="n">
         <v>6.29</v>
@@ -4927,10 +4927,10 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>16666.01</v>
+        <v>3030.18</v>
       </c>
       <c r="E125" t="n">
-        <v>2568</v>
+        <v>466.9</v>
       </c>
       <c r="F125" t="n">
         <v>6.49</v>
@@ -4963,10 +4963,10 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>16362.32</v>
+        <v>2974.97</v>
       </c>
       <c r="E126" t="n">
-        <v>2521.2</v>
+        <v>458.4</v>
       </c>
       <c r="F126" t="n">
         <v>6.49</v>
@@ -4999,10 +4999,10 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>15894.4</v>
+        <v>2889.89</v>
       </c>
       <c r="E127" t="n">
-        <v>2449.1</v>
+        <v>445.3</v>
       </c>
       <c r="F127" t="n">
         <v>6.49</v>
@@ -5035,10 +5035,10 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>16086.82</v>
+        <v>2924.88</v>
       </c>
       <c r="E128" t="n">
-        <v>3749.8</v>
+        <v>681.8</v>
       </c>
       <c r="F128" t="n">
         <v>4.29</v>
@@ -5071,10 +5071,10 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>16145.97</v>
+        <v>2935.63</v>
       </c>
       <c r="E129" t="n">
-        <v>3763.6</v>
+        <v>684.3</v>
       </c>
       <c r="F129" t="n">
         <v>4.29</v>
@@ -5107,10 +5107,10 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>16468.83</v>
+        <v>2994.33</v>
       </c>
       <c r="E130" t="n">
-        <v>3838.9</v>
+        <v>698</v>
       </c>
       <c r="F130" t="n">
         <v>4.29</v>
@@ -5143,10 +5143,10 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>15139.44</v>
+        <v>2752.63</v>
       </c>
       <c r="E131" t="n">
-        <v>3701.6</v>
+        <v>673</v>
       </c>
       <c r="F131" t="n">
         <v>4.09</v>
@@ -5179,10 +5179,10 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>14895.64</v>
+        <v>2708.3</v>
       </c>
       <c r="E132" t="n">
-        <v>3642</v>
+        <v>662.2</v>
       </c>
       <c r="F132" t="n">
         <v>4.09</v>
@@ -5215,10 +5215,10 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>14288.66</v>
+        <v>2597.94</v>
       </c>
       <c r="E133" t="n">
-        <v>3493.6</v>
+        <v>635.2</v>
       </c>
       <c r="F133" t="n">
         <v>4.09</v>
@@ -5251,10 +5251,10 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>12629.12</v>
+        <v>2296.2</v>
       </c>
       <c r="E134" t="n">
-        <v>4526.6</v>
+        <v>823</v>
       </c>
       <c r="F134" t="n">
         <v>2.79</v>
@@ -5287,10 +5287,10 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>12156.38</v>
+        <v>2210.25</v>
       </c>
       <c r="E135" t="n">
-        <v>4357.1</v>
+        <v>792.2</v>
       </c>
       <c r="F135" t="n">
         <v>2.79</v>
@@ -5323,10 +5323,10 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>12621.42</v>
+        <v>2294.8</v>
       </c>
       <c r="E136" t="n">
-        <v>4523.8</v>
+        <v>822.5</v>
       </c>
       <c r="F136" t="n">
         <v>2.79</v>
@@ -5359,10 +5359,10 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14576.22</v>
+        <v>2650.22</v>
       </c>
       <c r="E137" t="n">
-        <v>2317.4</v>
+        <v>421.3</v>
       </c>
       <c r="F137" t="n">
         <v>6.29</v>
@@ -5395,10 +5395,10 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>14206.73</v>
+        <v>2583.04</v>
       </c>
       <c r="E138" t="n">
-        <v>2258.6</v>
+        <v>410.7</v>
       </c>
       <c r="F138" t="n">
         <v>6.29</v>
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>14572.85</v>
+        <v>2649.61</v>
       </c>
       <c r="E139" t="n">
-        <v>2316.8</v>
+        <v>421.2</v>
       </c>
       <c r="F139" t="n">
         <v>6.29</v>
@@ -5467,10 +5467,10 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>15993.86</v>
+        <v>2907.97</v>
       </c>
       <c r="E140" t="n">
-        <v>2464.4</v>
+        <v>448.1</v>
       </c>
       <c r="F140" t="n">
         <v>6.49</v>
@@ -5503,10 +5503,10 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>16644.83</v>
+        <v>3026.33</v>
       </c>
       <c r="E141" t="n">
-        <v>2564.7</v>
+        <v>466.3</v>
       </c>
       <c r="F141" t="n">
         <v>6.49</v>
@@ -5539,10 +5539,10 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>16256.52</v>
+        <v>2955.73</v>
       </c>
       <c r="E142" t="n">
-        <v>2504.9</v>
+        <v>455.4</v>
       </c>
       <c r="F142" t="n">
         <v>6.49</v>
@@ -5575,10 +5575,10 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>16008.98</v>
+        <v>2910.72</v>
       </c>
       <c r="E143" t="n">
-        <v>3731.7</v>
+        <v>678.5</v>
       </c>
       <c r="F143" t="n">
         <v>4.29</v>
@@ -5611,10 +5611,10 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>17025.33</v>
+        <v>3095.51</v>
       </c>
       <c r="E144" t="n">
-        <v>3968.6</v>
+        <v>721.6</v>
       </c>
       <c r="F144" t="n">
         <v>4.29</v>
@@ -5647,10 +5647,10 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>16502.32</v>
+        <v>3000.42</v>
       </c>
       <c r="E145" t="n">
-        <v>3846.7</v>
+        <v>699.4</v>
       </c>
       <c r="F145" t="n">
         <v>4.29</v>
@@ -5683,10 +5683,10 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>14202.56</v>
+        <v>2582.28</v>
       </c>
       <c r="E146" t="n">
-        <v>3472.5</v>
+        <v>631.4</v>
       </c>
       <c r="F146" t="n">
         <v>4.09</v>
@@ -5719,10 +5719,10 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>14215.49</v>
+        <v>2584.63</v>
       </c>
       <c r="E147" t="n">
-        <v>3475.7</v>
+        <v>631.9</v>
       </c>
       <c r="F147" t="n">
         <v>4.09</v>
@@ -5755,10 +5755,10 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>14841.12</v>
+        <v>2698.38</v>
       </c>
       <c r="E148" t="n">
-        <v>3628.6</v>
+        <v>659.8</v>
       </c>
       <c r="F148" t="n">
         <v>4.09</v>
@@ -5791,10 +5791,10 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>11831.48</v>
+        <v>2151.18</v>
       </c>
       <c r="E149" t="n">
-        <v>4240.7</v>
+        <v>771</v>
       </c>
       <c r="F149" t="n">
         <v>2.79</v>
@@ -5827,10 +5827,10 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>12066.42</v>
+        <v>2193.89</v>
       </c>
       <c r="E150" t="n">
-        <v>4324.9</v>
+        <v>786.3</v>
       </c>
       <c r="F150" t="n">
         <v>2.79</v>
@@ -5863,10 +5863,10 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>11922.24</v>
+        <v>2167.68</v>
       </c>
       <c r="E151" t="n">
-        <v>4273.2</v>
+        <v>776.9</v>
       </c>
       <c r="F151" t="n">
         <v>2.79</v>
@@ -5899,10 +5899,10 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14565.28</v>
+        <v>2648.23</v>
       </c>
       <c r="E152" t="n">
-        <v>2315.6</v>
+        <v>421</v>
       </c>
       <c r="F152" t="n">
         <v>6.29</v>
@@ -5935,10 +5935,10 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>14638.6</v>
+        <v>2661.56</v>
       </c>
       <c r="E153" t="n">
-        <v>2327.3</v>
+        <v>423.1</v>
       </c>
       <c r="F153" t="n">
         <v>6.29</v>
@@ -5971,10 +5971,10 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>13974.08</v>
+        <v>2540.74</v>
       </c>
       <c r="E154" t="n">
-        <v>2221.6</v>
+        <v>403.9</v>
       </c>
       <c r="F154" t="n">
         <v>6.29</v>
@@ -6007,10 +6007,10 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>16082.2</v>
+        <v>2924.04</v>
       </c>
       <c r="E155" t="n">
-        <v>2478</v>
+        <v>450.5</v>
       </c>
       <c r="F155" t="n">
         <v>6.49</v>
@@ -6043,10 +6043,10 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>15863.36</v>
+        <v>2884.25</v>
       </c>
       <c r="E156" t="n">
-        <v>2444.3</v>
+        <v>444.4</v>
       </c>
       <c r="F156" t="n">
         <v>6.49</v>
@@ -6079,10 +6079,10 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>15961.59</v>
+        <v>2902.11</v>
       </c>
       <c r="E157" t="n">
-        <v>2459.4</v>
+        <v>447.2</v>
       </c>
       <c r="F157" t="n">
         <v>6.49</v>
@@ -6115,10 +6115,10 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>15988.35</v>
+        <v>2906.97</v>
       </c>
       <c r="E158" t="n">
-        <v>3726.9</v>
+        <v>677.6</v>
       </c>
       <c r="F158" t="n">
         <v>4.29</v>
@@ -6151,10 +6151,10 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>16890.2</v>
+        <v>3070.94</v>
       </c>
       <c r="E159" t="n">
-        <v>3937.1</v>
+        <v>715.8</v>
       </c>
       <c r="F159" t="n">
         <v>4.29</v>
@@ -6187,10 +6187,10 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>17101.06</v>
+        <v>3109.28</v>
       </c>
       <c r="E160" t="n">
-        <v>3986.3</v>
+        <v>724.8</v>
       </c>
       <c r="F160" t="n">
         <v>4.29</v>
@@ -6223,10 +6223,10 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>14062.93</v>
+        <v>2556.9</v>
       </c>
       <c r="E161" t="n">
-        <v>3438.4</v>
+        <v>625.2</v>
       </c>
       <c r="F161" t="n">
         <v>4.09</v>
@@ -6259,10 +6259,10 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>14740.33</v>
+        <v>2680.06</v>
       </c>
       <c r="E162" t="n">
-        <v>3604</v>
+        <v>655.3</v>
       </c>
       <c r="F162" t="n">
         <v>4.09</v>
@@ -6295,10 +6295,10 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>14930.38</v>
+        <v>2714.61</v>
       </c>
       <c r="E163" t="n">
-        <v>3650.5</v>
+        <v>663.7</v>
       </c>
       <c r="F163" t="n">
         <v>4.09</v>
@@ -6331,10 +6331,10 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>12064.66</v>
+        <v>2193.58</v>
       </c>
       <c r="E164" t="n">
-        <v>4324.3</v>
+        <v>786.2</v>
       </c>
       <c r="F164" t="n">
         <v>2.79</v>
@@ -6367,10 +6367,10 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>12558.4</v>
+        <v>2283.35</v>
       </c>
       <c r="E165" t="n">
-        <v>4501.2</v>
+        <v>818.4</v>
       </c>
       <c r="F165" t="n">
         <v>2.79</v>
@@ -6403,10 +6403,10 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>12405.98</v>
+        <v>2255.63</v>
       </c>
       <c r="E166" t="n">
-        <v>4446.6</v>
+        <v>808.5</v>
       </c>
       <c r="F166" t="n">
         <v>2.79</v>
@@ -6439,10 +6439,10 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>14436.62</v>
+        <v>2624.84</v>
       </c>
       <c r="E167" t="n">
-        <v>2295.2</v>
+        <v>417.3</v>
       </c>
       <c r="F167" t="n">
         <v>6.29</v>
@@ -6475,10 +6475,10 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>14342.37</v>
+        <v>2607.7</v>
       </c>
       <c r="E168" t="n">
-        <v>2280.2</v>
+        <v>414.6</v>
       </c>
       <c r="F168" t="n">
         <v>6.29</v>
@@ -6511,10 +6511,10 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>15405.93</v>
+        <v>2801.08</v>
       </c>
       <c r="E169" t="n">
-        <v>2449.3</v>
+        <v>445.3</v>
       </c>
       <c r="F169" t="n">
         <v>6.29</v>
@@ -6547,10 +6547,10 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>15761.81</v>
+        <v>2865.78</v>
       </c>
       <c r="E170" t="n">
-        <v>2428.6</v>
+        <v>441.6</v>
       </c>
       <c r="F170" t="n">
         <v>6.49</v>
@@ -6583,10 +6583,10 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>16067.97</v>
+        <v>2921.45</v>
       </c>
       <c r="E171" t="n">
-        <v>2475.8</v>
+        <v>450.1</v>
       </c>
       <c r="F171" t="n">
         <v>6.49</v>
@@ -6619,10 +6619,10 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>15536.79</v>
+        <v>2824.87</v>
       </c>
       <c r="E172" t="n">
-        <v>2394</v>
+        <v>435.3</v>
       </c>
       <c r="F172" t="n">
         <v>6.49</v>
@@ -6655,10 +6655,10 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>16415.62</v>
+        <v>2984.66</v>
       </c>
       <c r="E173" t="n">
-        <v>3826.5</v>
+        <v>695.7</v>
       </c>
       <c r="F173" t="n">
         <v>4.29</v>
@@ -6691,10 +6691,10 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>17084.81</v>
+        <v>3106.33</v>
       </c>
       <c r="E174" t="n">
-        <v>3982.5</v>
+        <v>724.1</v>
       </c>
       <c r="F174" t="n">
         <v>4.29</v>
@@ -6727,10 +6727,10 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>16519.69</v>
+        <v>3003.58</v>
       </c>
       <c r="E175" t="n">
-        <v>3850.7</v>
+        <v>700.1</v>
       </c>
       <c r="F175" t="n">
         <v>4.29</v>
@@ -6763,10 +6763,10 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>15172.86</v>
+        <v>2758.7</v>
       </c>
       <c r="E176" t="n">
-        <v>3709.7</v>
+        <v>674.5</v>
       </c>
       <c r="F176" t="n">
         <v>4.09</v>
@@ -6799,10 +6799,10 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>14339.65</v>
+        <v>2607.21</v>
       </c>
       <c r="E177" t="n">
-        <v>3506</v>
+        <v>637.5</v>
       </c>
       <c r="F177" t="n">
         <v>4.09</v>
@@ -6835,10 +6835,10 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>14627.07</v>
+        <v>2659.47</v>
       </c>
       <c r="E178" t="n">
-        <v>3576.3</v>
+        <v>650.2</v>
       </c>
       <c r="F178" t="n">
         <v>4.09</v>
@@ -6871,10 +6871,10 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>12629.09</v>
+        <v>2296.2</v>
       </c>
       <c r="E179" t="n">
-        <v>4526.6</v>
+        <v>823</v>
       </c>
       <c r="F179" t="n">
         <v>2.79</v>
@@ -6907,10 +6907,10 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>12225.18</v>
+        <v>2222.76</v>
       </c>
       <c r="E180" t="n">
-        <v>4381.8</v>
+        <v>796.7</v>
       </c>
       <c r="F180" t="n">
         <v>2.79</v>
@@ -6943,10 +6943,10 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>12059.44</v>
+        <v>2192.63</v>
       </c>
       <c r="E181" t="n">
-        <v>4322.4</v>
+        <v>785.9</v>
       </c>
       <c r="F181" t="n">
         <v>2.79</v>
@@ -6979,10 +6979,10 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>15837.7</v>
+        <v>2879.58</v>
       </c>
       <c r="E182" t="n">
-        <v>2517.9</v>
+        <v>457.8</v>
       </c>
       <c r="F182" t="n">
         <v>6.29</v>
@@ -7015,10 +7015,10 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>15526.04</v>
+        <v>2822.92</v>
       </c>
       <c r="E183" t="n">
-        <v>2468.4</v>
+        <v>448.8</v>
       </c>
       <c r="F183" t="n">
         <v>6.29</v>
@@ -7051,10 +7051,10 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>15395.01</v>
+        <v>2799.09</v>
       </c>
       <c r="E184" t="n">
-        <v>2447.5</v>
+        <v>445</v>
       </c>
       <c r="F184" t="n">
         <v>6.29</v>
@@ -7087,10 +7087,10 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>16515.88</v>
+        <v>3002.89</v>
       </c>
       <c r="E185" t="n">
-        <v>2544.8</v>
+        <v>462.7</v>
       </c>
       <c r="F185" t="n">
         <v>6.49</v>
@@ -7123,10 +7123,10 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>16155.21</v>
+        <v>2937.31</v>
       </c>
       <c r="E186" t="n">
-        <v>2489.2</v>
+        <v>452.6</v>
       </c>
       <c r="F186" t="n">
         <v>6.49</v>
@@ -7159,10 +7159,10 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>15695.02</v>
+        <v>2853.64</v>
       </c>
       <c r="E187" t="n">
-        <v>2418.3</v>
+        <v>439.7</v>
       </c>
       <c r="F187" t="n">
         <v>6.49</v>
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>17045.15</v>
+        <v>3099.12</v>
       </c>
       <c r="E188" t="n">
-        <v>3973.2</v>
+        <v>722.4</v>
       </c>
       <c r="F188" t="n">
         <v>4.29</v>
@@ -7231,10 +7231,10 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>16308.59</v>
+        <v>2965.2</v>
       </c>
       <c r="E189" t="n">
-        <v>3801.5</v>
+        <v>691.2</v>
       </c>
       <c r="F189" t="n">
         <v>4.29</v>
@@ -7267,10 +7267,10 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>15907.34</v>
+        <v>2892.24</v>
       </c>
       <c r="E190" t="n">
-        <v>3708</v>
+        <v>674.2</v>
       </c>
       <c r="F190" t="n">
         <v>4.29</v>
@@ -7303,10 +7303,10 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>14615.43</v>
+        <v>2657.35</v>
       </c>
       <c r="E191" t="n">
-        <v>3573.5</v>
+        <v>649.7</v>
       </c>
       <c r="F191" t="n">
         <v>4.09</v>
@@ -7339,10 +7339,10 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>14181.86</v>
+        <v>2578.52</v>
       </c>
       <c r="E192" t="n">
-        <v>3467.4</v>
+        <v>630.4</v>
       </c>
       <c r="F192" t="n">
         <v>4.09</v>
@@ -7375,10 +7375,10 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>14315.82</v>
+        <v>2602.88</v>
       </c>
       <c r="E193" t="n">
-        <v>3500.2</v>
+        <v>636.4</v>
       </c>
       <c r="F193" t="n">
         <v>4.09</v>
@@ -7411,10 +7411,10 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>12518.68</v>
+        <v>2276.12</v>
       </c>
       <c r="E194" t="n">
-        <v>4487</v>
+        <v>815.8</v>
       </c>
       <c r="F194" t="n">
         <v>2.79</v>
@@ -7447,10 +7447,10 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>11913.37</v>
+        <v>2166.07</v>
       </c>
       <c r="E195" t="n">
-        <v>4270</v>
+        <v>776.4</v>
       </c>
       <c r="F195" t="n">
         <v>2.79</v>
@@ -7483,10 +7483,10 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>12577.44</v>
+        <v>2286.81</v>
       </c>
       <c r="E196" t="n">
-        <v>4508</v>
+        <v>819.6</v>
       </c>
       <c r="F196" t="n">
         <v>2.79</v>
@@ -7519,10 +7519,10 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>15582.52</v>
+        <v>2833.19</v>
       </c>
       <c r="E197" t="n">
-        <v>2477.3</v>
+        <v>450.4</v>
       </c>
       <c r="F197" t="n">
         <v>6.29</v>
@@ -7555,10 +7555,10 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>15752.39</v>
+        <v>2864.07</v>
       </c>
       <c r="E198" t="n">
-        <v>2504.4</v>
+        <v>455.3</v>
       </c>
       <c r="F198" t="n">
         <v>6.29</v>
@@ -7591,10 +7591,10 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>15795.71</v>
+        <v>2871.95</v>
       </c>
       <c r="E199" t="n">
-        <v>2511.2</v>
+        <v>456.6</v>
       </c>
       <c r="F199" t="n">
         <v>6.29</v>
@@ -7627,10 +7627,10 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>15462.4</v>
+        <v>2811.35</v>
       </c>
       <c r="E200" t="n">
-        <v>2382.5</v>
+        <v>433.2</v>
       </c>
       <c r="F200" t="n">
         <v>6.49</v>
@@ -7663,10 +7663,10 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>15779.22</v>
+        <v>2868.95</v>
       </c>
       <c r="E201" t="n">
-        <v>2431.3</v>
+        <v>442.1</v>
       </c>
       <c r="F201" t="n">
         <v>6.49</v>
@@ -7699,10 +7699,10 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>15668.17</v>
+        <v>2848.76</v>
       </c>
       <c r="E202" t="n">
-        <v>2414.2</v>
+        <v>438.9</v>
       </c>
       <c r="F202" t="n">
         <v>6.49</v>
@@ -7735,10 +7735,10 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>16356.12</v>
+        <v>2973.84</v>
       </c>
       <c r="E203" t="n">
-        <v>3812.6</v>
+        <v>693.2</v>
       </c>
       <c r="F203" t="n">
         <v>4.29</v>
@@ -7771,10 +7771,10 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>16364.77</v>
+        <v>2975.41</v>
       </c>
       <c r="E204" t="n">
-        <v>3814.6</v>
+        <v>693.6</v>
       </c>
       <c r="F204" t="n">
         <v>4.29</v>
@@ -7807,10 +7807,10 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>16303.78</v>
+        <v>2964.32</v>
       </c>
       <c r="E205" t="n">
-        <v>3800.4</v>
+        <v>691</v>
       </c>
       <c r="F205" t="n">
         <v>4.29</v>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>14420.47</v>
+        <v>2621.9</v>
       </c>
       <c r="E206" t="n">
-        <v>3525.8</v>
+        <v>641.1</v>
       </c>
       <c r="F206" t="n">
         <v>4.09</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>14141.84</v>
+        <v>2571.24</v>
       </c>
       <c r="E207" t="n">
-        <v>3457.7</v>
+        <v>628.7</v>
       </c>
       <c r="F207" t="n">
         <v>4.09</v>
@@ -7915,10 +7915,10 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>14066.36</v>
+        <v>2557.52</v>
       </c>
       <c r="E208" t="n">
-        <v>3439.2</v>
+        <v>625.3</v>
       </c>
       <c r="F208" t="n">
         <v>4.09</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>11983.45</v>
+        <v>2178.81</v>
       </c>
       <c r="E209" t="n">
-        <v>4295.1</v>
+        <v>780.9</v>
       </c>
       <c r="F209" t="n">
         <v>2.79</v>
@@ -7987,10 +7987,10 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>12528.05</v>
+        <v>2277.83</v>
       </c>
       <c r="E210" t="n">
-        <v>4490.3</v>
+        <v>816.4</v>
       </c>
       <c r="F210" t="n">
         <v>2.79</v>
@@ -8023,10 +8023,10 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>12758.01</v>
+        <v>2319.64</v>
       </c>
       <c r="E211" t="n">
-        <v>4572.8</v>
+        <v>831.4</v>
       </c>
       <c r="F211" t="n">
         <v>2.79</v>
@@ -8059,10 +8059,10 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>16787.69</v>
+        <v>3052.31</v>
       </c>
       <c r="E212" t="n">
-        <v>2668.9</v>
+        <v>485.3</v>
       </c>
       <c r="F212" t="n">
         <v>6.29</v>
@@ -8095,10 +8095,10 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>15897.93</v>
+        <v>2890.53</v>
       </c>
       <c r="E213" t="n">
-        <v>2527.5</v>
+        <v>459.5</v>
       </c>
       <c r="F213" t="n">
         <v>6.29</v>
@@ -8131,10 +8131,10 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>16638.01</v>
+        <v>3025.09</v>
       </c>
       <c r="E214" t="n">
-        <v>2645.2</v>
+        <v>480.9</v>
       </c>
       <c r="F214" t="n">
         <v>6.29</v>
@@ -8167,10 +8167,10 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>15464.16</v>
+        <v>2811.67</v>
       </c>
       <c r="E215" t="n">
-        <v>2382.8</v>
+        <v>433.2</v>
       </c>
       <c r="F215" t="n">
         <v>6.49</v>
@@ -8203,10 +8203,10 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>16409.95</v>
+        <v>2983.63</v>
       </c>
       <c r="E216" t="n">
-        <v>2528.5</v>
+        <v>459.7</v>
       </c>
       <c r="F216" t="n">
         <v>6.49</v>
@@ -8239,10 +8239,10 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>16447.26</v>
+        <v>2990.41</v>
       </c>
       <c r="E217" t="n">
-        <v>2534.2</v>
+        <v>460.8</v>
       </c>
       <c r="F217" t="n">
         <v>6.49</v>
@@ -8275,10 +8275,10 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>16651.82</v>
+        <v>3027.6</v>
       </c>
       <c r="E218" t="n">
-        <v>3881.5</v>
+        <v>705.7</v>
       </c>
       <c r="F218" t="n">
         <v>4.29</v>
@@ -8311,10 +8311,10 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>16988.03</v>
+        <v>3088.73</v>
       </c>
       <c r="E219" t="n">
-        <v>3959.9</v>
+        <v>720</v>
       </c>
       <c r="F219" t="n">
         <v>4.29</v>
@@ -8347,10 +8347,10 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>15985.18</v>
+        <v>2906.4</v>
       </c>
       <c r="E220" t="n">
-        <v>3726.1</v>
+        <v>677.5</v>
       </c>
       <c r="F220" t="n">
         <v>4.29</v>
@@ -8383,10 +8383,10 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>14359.64</v>
+        <v>2610.84</v>
       </c>
       <c r="E221" t="n">
-        <v>3510.9</v>
+        <v>638.3</v>
       </c>
       <c r="F221" t="n">
         <v>4.09</v>
@@ -8419,10 +8419,10 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>14521.36</v>
+        <v>2640.25</v>
       </c>
       <c r="E222" t="n">
-        <v>3550.5</v>
+        <v>645.5</v>
       </c>
       <c r="F222" t="n">
         <v>4.09</v>
@@ -8455,10 +8455,10 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>14086.54</v>
+        <v>2561.19</v>
       </c>
       <c r="E223" t="n">
-        <v>3444.1</v>
+        <v>626.2</v>
       </c>
       <c r="F223" t="n">
         <v>4.09</v>
@@ -8491,10 +8491,10 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>12225.14</v>
+        <v>2222.75</v>
       </c>
       <c r="E224" t="n">
-        <v>4381.8</v>
+        <v>796.7</v>
       </c>
       <c r="F224" t="n">
         <v>2.79</v>
@@ -8527,10 +8527,10 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>12045.42</v>
+        <v>2190.08</v>
       </c>
       <c r="E225" t="n">
-        <v>4317.4</v>
+        <v>785</v>
       </c>
       <c r="F225" t="n">
         <v>2.79</v>
@@ -8563,10 +8563,10 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>12170.66</v>
+        <v>2212.85</v>
       </c>
       <c r="E226" t="n">
-        <v>4362.2</v>
+        <v>793.1</v>
       </c>
       <c r="F226" t="n">
         <v>2.79</v>
@@ -8599,10 +8599,10 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>16960.85</v>
+        <v>3083.79</v>
       </c>
       <c r="E227" t="n">
-        <v>2696.5</v>
+        <v>490.3</v>
       </c>
       <c r="F227" t="n">
         <v>6.29</v>
@@ -8635,10 +8635,10 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>17947.57</v>
+        <v>3263.19</v>
       </c>
       <c r="E228" t="n">
-        <v>2853.3</v>
+        <v>518.8</v>
       </c>
       <c r="F228" t="n">
         <v>6.29</v>
@@ -8671,10 +8671,10 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>17691.5</v>
+        <v>3216.64</v>
       </c>
       <c r="E229" t="n">
-        <v>2812.6</v>
+        <v>511.4</v>
       </c>
       <c r="F229" t="n">
         <v>6.29</v>
@@ -8707,10 +8707,10 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>16663.62</v>
+        <v>3029.75</v>
       </c>
       <c r="E230" t="n">
-        <v>2567.6</v>
+        <v>466.8</v>
       </c>
       <c r="F230" t="n">
         <v>6.49</v>
@@ -8743,10 +8743,10 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>16497.26</v>
+        <v>2999.5</v>
       </c>
       <c r="E231" t="n">
-        <v>2542</v>
+        <v>462.2</v>
       </c>
       <c r="F231" t="n">
         <v>6.49</v>
@@ -8779,10 +8779,10 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>15602.85</v>
+        <v>2836.88</v>
       </c>
       <c r="E232" t="n">
-        <v>2404.1</v>
+        <v>437.1</v>
       </c>
       <c r="F232" t="n">
         <v>6.49</v>
@@ -8815,10 +8815,10 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>16551.46</v>
+        <v>3009.36</v>
       </c>
       <c r="E233" t="n">
-        <v>3858.1</v>
+        <v>701.5</v>
       </c>
       <c r="F233" t="n">
         <v>4.29</v>
@@ -8851,10 +8851,10 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>16080.44</v>
+        <v>2923.72</v>
       </c>
       <c r="E234" t="n">
-        <v>3748.4</v>
+        <v>681.5</v>
       </c>
       <c r="F234" t="n">
         <v>4.29</v>
@@ -8887,10 +8887,10 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>16936.98</v>
+        <v>3079.45</v>
       </c>
       <c r="E235" t="n">
-        <v>3948</v>
+        <v>717.8</v>
       </c>
       <c r="F235" t="n">
         <v>4.29</v>
@@ -8923,10 +8923,10 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>14720.2</v>
+        <v>2676.4</v>
       </c>
       <c r="E236" t="n">
-        <v>3599.1</v>
+        <v>654.4</v>
       </c>
       <c r="F236" t="n">
         <v>4.09</v>
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>14345.05</v>
+        <v>2608.19</v>
       </c>
       <c r="E237" t="n">
-        <v>3507.3</v>
+        <v>637.7</v>
       </c>
       <c r="F237" t="n">
         <v>4.09</v>
@@ -8995,10 +8995,10 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>15124.27</v>
+        <v>2749.87</v>
       </c>
       <c r="E238" t="n">
-        <v>3697.9</v>
+        <v>672.3</v>
       </c>
       <c r="F238" t="n">
         <v>4.09</v>
@@ -9031,10 +9031,10 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>11898.08</v>
+        <v>2163.29</v>
       </c>
       <c r="E239" t="n">
-        <v>4264.5</v>
+        <v>775.4</v>
       </c>
       <c r="F239" t="n">
         <v>2.79</v>
@@ -9067,10 +9067,10 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>12338.72</v>
+        <v>2243.4</v>
       </c>
       <c r="E240" t="n">
-        <v>4422.5</v>
+        <v>804.1</v>
       </c>
       <c r="F240" t="n">
         <v>2.79</v>
@@ -9103,10 +9103,10 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>12493.08</v>
+        <v>2271.47</v>
       </c>
       <c r="E241" t="n">
-        <v>4477.8</v>
+        <v>814.1</v>
       </c>
       <c r="F241" t="n">
         <v>2.79</v>

</xml_diff>

<commit_message>
Fix share score: model full IRI market in build_iri()
Share score was 2/100 for strong_promo because market_share_dollars
was computed from this retailer only. With IRI_MULT=5.5, a single-
retailer promo swing of 14.8pp collapsed to ~1.7% share retention
after the promo, giving a near-zero score.

Fix: incorporate other retailers (4.5× baseline) into both the
numerator and denominator of market_share_* columns. Each brand's
other-retailer volume is split equally across its SKUs so brand-level
shares sum correctly. Summit gains a spillover multiplier in late
post-promo weeks (W13-16) to model permanent brand conversion.

Results: strong_promo share 39/100 (was 2), retention 38.7%,
3.05pp gain. Grades unchanged: A / B / C. Zero validation warnings.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stella/test_fixtures/inventory_risk/iri_data.xlsx
+++ b/stella/test_fixtures/inventory_risk/iri_data.xlsx
@@ -508,10 +508,10 @@
         <v>6.29</v>
       </c>
       <c r="G2" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0746</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0519</v>
+        <v>0.0534</v>
       </c>
       <c r="I2" t="n">
         <v>92</v>
@@ -544,10 +544,10 @@
         <v>6.29</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0746</v>
+        <v>0.075</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0535</v>
+        <v>0.0537</v>
       </c>
       <c r="I3" t="n">
         <v>91</v>
@@ -580,10 +580,10 @@
         <v>6.29</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0779</v>
+        <v>0.0756</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0558</v>
+        <v>0.0541</v>
       </c>
       <c r="I4" t="n">
         <v>91</v>
@@ -616,10 +616,10 @@
         <v>6.49</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0673</v>
+        <v>0.0693</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0468</v>
+        <v>0.0481</v>
       </c>
       <c r="I5" t="n">
         <v>91</v>
@@ -652,10 +652,10 @@
         <v>6.49</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0712</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0495</v>
+        <v>0.0486</v>
       </c>
       <c r="I6" t="n">
         <v>90</v>
@@ -688,10 +688,10 @@
         <v>6.49</v>
       </c>
       <c r="G7" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0476</v>
+        <v>0.0482</v>
       </c>
       <c r="I7" t="n">
         <v>90</v>
@@ -724,10 +724,10 @@
         <v>4.29</v>
       </c>
       <c r="G8" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.0721</v>
       </c>
       <c r="H8" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0757</v>
       </c>
       <c r="I8" t="n">
         <v>90</v>
@@ -760,10 +760,10 @@
         <v>4.29</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0732</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>0.077</v>
+        <v>0.0756</v>
       </c>
       <c r="I9" t="n">
         <v>91</v>
@@ -796,10 +796,10 @@
         <v>4.29</v>
       </c>
       <c r="G10" t="n">
-        <v>0.074</v>
+        <v>0.0721</v>
       </c>
       <c r="H10" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0757</v>
       </c>
       <c r="I10" t="n">
         <v>89</v>
@@ -832,10 +832,10 @@
         <v>4.09</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0621</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0696</v>
       </c>
       <c r="I11" t="n">
         <v>92</v>
@@ -868,10 +868,10 @@
         <v>4.09</v>
       </c>
       <c r="G12" t="n">
-        <v>0.06370000000000001</v>
+        <v>0.0635</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0703</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I12" t="n">
         <v>91</v>
@@ -904,10 +904,10 @@
         <v>4.09</v>
       </c>
       <c r="G13" t="n">
-        <v>0.065</v>
+        <v>0.0638</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0717</v>
+        <v>0.0702</v>
       </c>
       <c r="I13" t="n">
         <v>89</v>
@@ -940,10 +940,10 @@
         <v>2.79</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0523</v>
+        <v>0.0531</v>
       </c>
       <c r="H14" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.0857</v>
       </c>
       <c r="I14" t="n">
         <v>90</v>
@@ -976,10 +976,10 @@
         <v>2.79</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0522</v>
+        <v>0.0531</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0844</v>
+        <v>0.0857</v>
       </c>
       <c r="I15" t="n">
         <v>88</v>
@@ -1012,10 +1012,10 @@
         <v>2.79</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0514</v>
+        <v>0.0529</v>
       </c>
       <c r="H16" t="n">
-        <v>0.083</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="I16" t="n">
         <v>92</v>
@@ -1048,10 +1048,10 @@
         <v>6.29</v>
       </c>
       <c r="G17" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0756</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0556</v>
+        <v>0.0541</v>
       </c>
       <c r="I17" t="n">
         <v>92</v>
@@ -1084,10 +1084,10 @@
         <v>6.29</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0779</v>
+        <v>0.0756</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0557</v>
+        <v>0.0541</v>
       </c>
       <c r="I18" t="n">
         <v>91</v>
@@ -1120,10 +1120,10 @@
         <v>6.29</v>
       </c>
       <c r="G19" t="n">
-        <v>0.07439999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0532</v>
+        <v>0.0537</v>
       </c>
       <c r="I19" t="n">
         <v>90</v>
@@ -1156,10 +1156,10 @@
         <v>6.49</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0682</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0472</v>
+        <v>0.0482</v>
       </c>
       <c r="I20" t="n">
         <v>91</v>
@@ -1192,10 +1192,10 @@
         <v>6.49</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0684</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0474</v>
+        <v>0.0482</v>
       </c>
       <c r="I21" t="n">
         <v>90</v>
@@ -1228,10 +1228,10 @@
         <v>6.49</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0677</v>
+        <v>0.0694</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0469</v>
+        <v>0.0481</v>
       </c>
       <c r="I22" t="n">
         <v>89</v>
@@ -1264,10 +1264,10 @@
         <v>4.29</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0698</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0732</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="I23" t="n">
         <v>90</v>
@@ -1300,10 +1300,10 @@
         <v>4.29</v>
       </c>
       <c r="G24" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0713</v>
       </c>
       <c r="H24" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="I24" t="n">
         <v>88</v>
@@ -1336,10 +1336,10 @@
         <v>4.29</v>
       </c>
       <c r="G25" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.0723</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0784</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="I25" t="n">
         <v>91</v>
@@ -1372,10 +1372,10 @@
         <v>4.09</v>
       </c>
       <c r="G26" t="n">
-        <v>0.0616</v>
+        <v>0.0631</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0677</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="I26" t="n">
         <v>89</v>
@@ -1408,10 +1408,10 @@
         <v>4.09</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0619</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="H27" t="n">
-        <v>0.068</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="I27" t="n">
         <v>88</v>
@@ -1444,10 +1444,10 @@
         <v>4.09</v>
       </c>
       <c r="G28" t="n">
-        <v>0.0654</v>
+        <v>0.0638</v>
       </c>
       <c r="H28" t="n">
-        <v>0.07190000000000001</v>
+        <v>0.0703</v>
       </c>
       <c r="I28" t="n">
         <v>89</v>
@@ -1480,10 +1480,10 @@
         <v>2.79</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0539</v>
+        <v>0.0534</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0868</v>
+        <v>0.0862</v>
       </c>
       <c r="I29" t="n">
         <v>92</v>
@@ -1516,10 +1516,10 @@
         <v>2.79</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0547</v>
+        <v>0.0535</v>
       </c>
       <c r="H30" t="n">
-        <v>0.0881</v>
+        <v>0.0864</v>
       </c>
       <c r="I30" t="n">
         <v>89</v>
@@ -1552,10 +1552,10 @@
         <v>2.79</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0541</v>
+        <v>0.0534</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0871</v>
+        <v>0.0862</v>
       </c>
       <c r="I31" t="n">
         <v>91</v>
@@ -1588,10 +1588,10 @@
         <v>6.29</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0772</v>
+        <v>0.0755</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0553</v>
+        <v>0.054</v>
       </c>
       <c r="I32" t="n">
         <v>91</v>
@@ -1624,10 +1624,10 @@
         <v>6.29</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0725</v>
+        <v>0.0746</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0519</v>
+        <v>0.0534</v>
       </c>
       <c r="I33" t="n">
         <v>91</v>
@@ -1660,10 +1660,10 @@
         <v>6.29</v>
       </c>
       <c r="G34" t="n">
-        <v>0.0767</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="H34" t="n">
-        <v>0.0549</v>
+        <v>0.054</v>
       </c>
       <c r="I34" t="n">
         <v>91</v>
@@ -1696,10 +1696,10 @@
         <v>6.49</v>
       </c>
       <c r="G35" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0476</v>
+        <v>0.0482</v>
       </c>
       <c r="I35" t="n">
         <v>88</v>
@@ -1732,10 +1732,10 @@
         <v>6.49</v>
       </c>
       <c r="G36" t="n">
-        <v>0.06809999999999999</v>
+        <v>0.0694</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0473</v>
+        <v>0.0482</v>
       </c>
       <c r="I36" t="n">
         <v>90</v>
@@ -1768,10 +1768,10 @@
         <v>6.49</v>
       </c>
       <c r="G37" t="n">
-        <v>0.0708</v>
+        <v>0.0699</v>
       </c>
       <c r="H37" t="n">
-        <v>0.0491</v>
+        <v>0.0485</v>
       </c>
       <c r="I37" t="n">
         <v>90</v>
@@ -1804,10 +1804,10 @@
         <v>4.29</v>
       </c>
       <c r="G38" t="n">
-        <v>0.074</v>
+        <v>0.0721</v>
       </c>
       <c r="H38" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0757</v>
       </c>
       <c r="I38" t="n">
         <v>88</v>
@@ -1840,10 +1840,10 @@
         <v>4.29</v>
       </c>
       <c r="G39" t="n">
-        <v>0.07049999999999999</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>0.074</v>
+        <v>0.075</v>
       </c>
       <c r="I39" t="n">
         <v>89</v>
@@ -1876,10 +1876,10 @@
         <v>4.29</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0721</v>
+        <v>0.0718</v>
       </c>
       <c r="H40" t="n">
-        <v>0.0757</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="I40" t="n">
         <v>90</v>
@@ -1912,10 +1912,10 @@
         <v>4.09</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0624</v>
+        <v>0.0633</v>
       </c>
       <c r="H41" t="n">
-        <v>0.0687</v>
+        <v>0.0697</v>
       </c>
       <c r="I41" t="n">
         <v>91</v>
@@ -1948,10 +1948,10 @@
         <v>4.09</v>
       </c>
       <c r="G42" t="n">
-        <v>0.06370000000000001</v>
+        <v>0.0635</v>
       </c>
       <c r="H42" t="n">
-        <v>0.0702</v>
+        <v>0.0699</v>
       </c>
       <c r="I42" t="n">
         <v>89</v>
@@ -1984,10 +1984,10 @@
         <v>4.09</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0641</v>
+        <v>0.0636</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0706</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I43" t="n">
         <v>92</v>
@@ -2020,10 +2020,10 @@
         <v>2.79</v>
       </c>
       <c r="G44" t="n">
-        <v>0.0537</v>
+        <v>0.0534</v>
       </c>
       <c r="H44" t="n">
-        <v>0.0868</v>
+        <v>0.0862</v>
       </c>
       <c r="I44" t="n">
         <v>90</v>
@@ -2056,10 +2056,10 @@
         <v>2.79</v>
       </c>
       <c r="G45" t="n">
-        <v>0.0538</v>
+        <v>0.0534</v>
       </c>
       <c r="H45" t="n">
-        <v>0.0868</v>
+        <v>0.0862</v>
       </c>
       <c r="I45" t="n">
         <v>91</v>
@@ -2092,10 +2092,10 @@
         <v>2.79</v>
       </c>
       <c r="G46" t="n">
-        <v>0.0517</v>
+        <v>0.053</v>
       </c>
       <c r="H46" t="n">
-        <v>0.0835</v>
+        <v>0.0856</v>
       </c>
       <c r="I46" t="n">
         <v>90</v>
@@ -2128,10 +2128,10 @@
         <v>6.29</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0746</v>
+        <v>0.075</v>
       </c>
       <c r="H47" t="n">
-        <v>0.0534</v>
+        <v>0.0537</v>
       </c>
       <c r="I47" t="n">
         <v>88</v>
@@ -2164,10 +2164,10 @@
         <v>6.29</v>
       </c>
       <c r="G48" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0751</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0539</v>
+        <v>0.0538</v>
       </c>
       <c r="I48" t="n">
         <v>89</v>
@@ -2200,10 +2200,10 @@
         <v>6.29</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0772</v>
+        <v>0.0755</v>
       </c>
       <c r="H49" t="n">
-        <v>0.0552</v>
+        <v>0.054</v>
       </c>
       <c r="I49" t="n">
         <v>88</v>
@@ -2236,10 +2236,10 @@
         <v>6.49</v>
       </c>
       <c r="G50" t="n">
-        <v>0.0692</v>
+        <v>0.0696</v>
       </c>
       <c r="H50" t="n">
-        <v>0.048</v>
+        <v>0.0483</v>
       </c>
       <c r="I50" t="n">
         <v>88</v>
@@ -2272,10 +2272,10 @@
         <v>6.49</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0694</v>
+        <v>0.0697</v>
       </c>
       <c r="H51" t="n">
-        <v>0.0482</v>
+        <v>0.0483</v>
       </c>
       <c r="I51" t="n">
         <v>90</v>
@@ -2311,7 +2311,7 @@
         <v>0.0698</v>
       </c>
       <c r="H52" t="n">
-        <v>0.0485</v>
+        <v>0.0484</v>
       </c>
       <c r="I52" t="n">
         <v>91</v>
@@ -2344,10 +2344,10 @@
         <v>4.29</v>
       </c>
       <c r="G53" t="n">
-        <v>0.0726</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="H53" t="n">
-        <v>0.0762</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="I53" t="n">
         <v>91</v>
@@ -2380,10 +2380,10 @@
         <v>4.29</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0688</v>
+        <v>0.0712</v>
       </c>
       <c r="H54" t="n">
-        <v>0.0722</v>
+        <v>0.0747</v>
       </c>
       <c r="I54" t="n">
         <v>88</v>
@@ -2416,10 +2416,10 @@
         <v>4.29</v>
       </c>
       <c r="G55" t="n">
-        <v>0.0713</v>
+        <v>0.0716</v>
       </c>
       <c r="H55" t="n">
-        <v>0.07489999999999999</v>
+        <v>0.0752</v>
       </c>
       <c r="I55" t="n">
         <v>90</v>
@@ -2452,10 +2452,10 @@
         <v>4.09</v>
       </c>
       <c r="G56" t="n">
-        <v>0.063</v>
+        <v>0.0634</v>
       </c>
       <c r="H56" t="n">
-        <v>0.0693</v>
+        <v>0.0698</v>
       </c>
       <c r="I56" t="n">
         <v>88</v>
@@ -2488,10 +2488,10 @@
         <v>4.09</v>
       </c>
       <c r="G57" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0638</v>
       </c>
       <c r="H57" t="n">
-        <v>0.0718</v>
+        <v>0.0702</v>
       </c>
       <c r="I57" t="n">
         <v>92</v>
@@ -2524,10 +2524,10 @@
         <v>4.09</v>
       </c>
       <c r="G58" t="n">
-        <v>0.063</v>
+        <v>0.0634</v>
       </c>
       <c r="H58" t="n">
-        <v>0.0694</v>
+        <v>0.0698</v>
       </c>
       <c r="I58" t="n">
         <v>88</v>
@@ -2560,10 +2560,10 @@
         <v>2.79</v>
       </c>
       <c r="G59" t="n">
-        <v>0.0528</v>
+        <v>0.0532</v>
       </c>
       <c r="H59" t="n">
-        <v>0.0852</v>
+        <v>0.0859</v>
       </c>
       <c r="I59" t="n">
         <v>91</v>
@@ -2596,10 +2596,10 @@
         <v>2.79</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0549</v>
+        <v>0.0536</v>
       </c>
       <c r="H60" t="n">
-        <v>0.0886</v>
+        <v>0.08649999999999999</v>
       </c>
       <c r="I60" t="n">
         <v>89</v>
@@ -2632,10 +2632,10 @@
         <v>2.79</v>
       </c>
       <c r="G61" t="n">
-        <v>0.0527</v>
+        <v>0.0532</v>
       </c>
       <c r="H61" t="n">
-        <v>0.0851</v>
+        <v>0.0859</v>
       </c>
       <c r="I61" t="n">
         <v>91</v>
@@ -2668,10 +2668,10 @@
         <v>5.04</v>
       </c>
       <c r="G62" t="n">
-        <v>0.1081</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="H62" t="n">
-        <v>0.0939</v>
+        <v>0.0619</v>
       </c>
       <c r="I62" t="n">
         <v>90</v>
@@ -2704,10 +2704,10 @@
         <v>5.04</v>
       </c>
       <c r="G63" t="n">
-        <v>0.1111</v>
+        <v>0.0822</v>
       </c>
       <c r="H63" t="n">
-        <v>0.0965</v>
+        <v>0.0624</v>
       </c>
       <c r="I63" t="n">
         <v>91</v>
@@ -2740,10 +2740,10 @@
         <v>5.04</v>
       </c>
       <c r="G64" t="n">
-        <v>0.1065</v>
+        <v>0.0813</v>
       </c>
       <c r="H64" t="n">
-        <v>0.0925</v>
+        <v>0.0616</v>
       </c>
       <c r="I64" t="n">
         <v>92</v>
@@ -2776,10 +2776,10 @@
         <v>6.49</v>
       </c>
       <c r="G65" t="n">
-        <v>0.0586</v>
+        <v>0.0675</v>
       </c>
       <c r="H65" t="n">
-        <v>0.0395</v>
+        <v>0.0466</v>
       </c>
       <c r="I65" t="n">
         <v>92</v>
@@ -2812,10 +2812,10 @@
         <v>6.49</v>
       </c>
       <c r="G66" t="n">
-        <v>0.0568</v>
+        <v>0.0672</v>
       </c>
       <c r="H66" t="n">
-        <v>0.0383</v>
+        <v>0.0464</v>
       </c>
       <c r="I66" t="n">
         <v>89</v>
@@ -2848,10 +2848,10 @@
         <v>6.49</v>
       </c>
       <c r="G67" t="n">
-        <v>0.0579</v>
+        <v>0.0674</v>
       </c>
       <c r="H67" t="n">
-        <v>0.0391</v>
+        <v>0.0465</v>
       </c>
       <c r="I67" t="n">
         <v>90</v>
@@ -2884,10 +2884,10 @@
         <v>4.29</v>
       </c>
       <c r="G68" t="n">
-        <v>0.064</v>
+        <v>0.0702</v>
       </c>
       <c r="H68" t="n">
-        <v>0.0653</v>
+        <v>0.0733</v>
       </c>
       <c r="I68" t="n">
         <v>92</v>
@@ -2920,10 +2920,10 @@
         <v>4.29</v>
       </c>
       <c r="G69" t="n">
-        <v>0.0648</v>
+        <v>0.0703</v>
       </c>
       <c r="H69" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="I69" t="n">
         <v>89</v>
@@ -2956,10 +2956,10 @@
         <v>4.29</v>
       </c>
       <c r="G70" t="n">
-        <v>0.0609</v>
+        <v>0.0696</v>
       </c>
       <c r="H70" t="n">
-        <v>0.0621</v>
+        <v>0.0726</v>
       </c>
       <c r="I70" t="n">
         <v>90</v>
@@ -2992,10 +2992,10 @@
         <v>4.09</v>
       </c>
       <c r="G71" t="n">
-        <v>0.0548</v>
+        <v>0.0618</v>
       </c>
       <c r="H71" t="n">
-        <v>0.0586</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="I71" t="n">
         <v>92</v>
@@ -3028,10 +3028,10 @@
         <v>4.09</v>
       </c>
       <c r="G72" t="n">
-        <v>0.0546</v>
+        <v>0.0617</v>
       </c>
       <c r="H72" t="n">
-        <v>0.0584</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="I72" t="n">
         <v>92</v>
@@ -3064,10 +3064,10 @@
         <v>4.09</v>
       </c>
       <c r="G73" t="n">
-        <v>0.0546</v>
+        <v>0.0617</v>
       </c>
       <c r="H73" t="n">
-        <v>0.0585</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="I73" t="n">
         <v>92</v>
@@ -3100,10 +3100,10 @@
         <v>2.79</v>
       </c>
       <c r="G74" t="n">
-        <v>0.048</v>
+        <v>0.0523</v>
       </c>
       <c r="H74" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0839</v>
       </c>
       <c r="I74" t="n">
         <v>91</v>
@@ -3136,10 +3136,10 @@
         <v>2.79</v>
       </c>
       <c r="G75" t="n">
-        <v>0.0496</v>
+        <v>0.0526</v>
       </c>
       <c r="H75" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0844</v>
       </c>
       <c r="I75" t="n">
         <v>89</v>
@@ -3172,10 +3172,10 @@
         <v>2.79</v>
       </c>
       <c r="G76" t="n">
-        <v>0.0496</v>
+        <v>0.0526</v>
       </c>
       <c r="H76" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0844</v>
       </c>
       <c r="I76" t="n">
         <v>89</v>
@@ -3208,10 +3208,10 @@
         <v>5.04</v>
       </c>
       <c r="G77" t="n">
-        <v>0.1101</v>
+        <v>0.082</v>
       </c>
       <c r="H77" t="n">
-        <v>0.0958</v>
+        <v>0.0622</v>
       </c>
       <c r="I77" t="n">
         <v>87</v>
@@ -3244,10 +3244,10 @@
         <v>5.04</v>
       </c>
       <c r="G78" t="n">
-        <v>0.1102</v>
+        <v>0.082</v>
       </c>
       <c r="H78" t="n">
-        <v>0.0959</v>
+        <v>0.0622</v>
       </c>
       <c r="I78" t="n">
         <v>89</v>
@@ -3280,10 +3280,10 @@
         <v>5.04</v>
       </c>
       <c r="G79" t="n">
-        <v>0.1097</v>
+        <v>0.0819</v>
       </c>
       <c r="H79" t="n">
-        <v>0.0955</v>
+        <v>0.0621</v>
       </c>
       <c r="I79" t="n">
         <v>88</v>
@@ -3316,10 +3316,10 @@
         <v>6.49</v>
       </c>
       <c r="G80" t="n">
-        <v>0.0578</v>
+        <v>0.0674</v>
       </c>
       <c r="H80" t="n">
-        <v>0.0391</v>
+        <v>0.0465</v>
       </c>
       <c r="I80" t="n">
         <v>91</v>
@@ -3352,10 +3352,10 @@
         <v>6.49</v>
       </c>
       <c r="G81" t="n">
-        <v>0.0568</v>
+        <v>0.0672</v>
       </c>
       <c r="H81" t="n">
-        <v>0.0384</v>
+        <v>0.0464</v>
       </c>
       <c r="I81" t="n">
         <v>89</v>
@@ -3388,10 +3388,10 @@
         <v>6.49</v>
       </c>
       <c r="G82" t="n">
-        <v>0.0583</v>
+        <v>0.0675</v>
       </c>
       <c r="H82" t="n">
-        <v>0.0394</v>
+        <v>0.0466</v>
       </c>
       <c r="I82" t="n">
         <v>88</v>
@@ -3424,10 +3424,10 @@
         <v>4.29</v>
       </c>
       <c r="G83" t="n">
-        <v>0.0619</v>
+        <v>0.0698</v>
       </c>
       <c r="H83" t="n">
-        <v>0.0633</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="I83" t="n">
         <v>88</v>
@@ -3460,10 +3460,10 @@
         <v>4.29</v>
       </c>
       <c r="G84" t="n">
-        <v>0.0619</v>
+        <v>0.0698</v>
       </c>
       <c r="H84" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="I84" t="n">
         <v>90</v>
@@ -3496,10 +3496,10 @@
         <v>4.29</v>
       </c>
       <c r="G85" t="n">
-        <v>0.0608</v>
+        <v>0.0696</v>
       </c>
       <c r="H85" t="n">
-        <v>0.0622</v>
+        <v>0.0727</v>
       </c>
       <c r="I85" t="n">
         <v>88</v>
@@ -3532,10 +3532,10 @@
         <v>4.09</v>
       </c>
       <c r="G86" t="n">
-        <v>0.0547</v>
+        <v>0.0618</v>
       </c>
       <c r="H86" t="n">
-        <v>0.0587</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="I86" t="n">
         <v>92</v>
@@ -3568,10 +3568,10 @@
         <v>4.09</v>
       </c>
       <c r="G87" t="n">
-        <v>0.0577</v>
+        <v>0.0623</v>
       </c>
       <c r="H87" t="n">
-        <v>0.0618</v>
+        <v>0.0683</v>
       </c>
       <c r="I87" t="n">
         <v>88</v>
@@ -3604,10 +3604,10 @@
         <v>4.09</v>
       </c>
       <c r="G88" t="n">
-        <v>0.0559</v>
+        <v>0.062</v>
       </c>
       <c r="H88" t="n">
-        <v>0.0599</v>
+        <v>0.0679</v>
       </c>
       <c r="I88" t="n">
         <v>91</v>
@@ -3640,10 +3640,10 @@
         <v>2.79</v>
       </c>
       <c r="G89" t="n">
-        <v>0.047</v>
+        <v>0.0521</v>
       </c>
       <c r="H89" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="I89" t="n">
         <v>90</v>
@@ -3676,10 +3676,10 @@
         <v>2.79</v>
       </c>
       <c r="G90" t="n">
-        <v>0.0491</v>
+        <v>0.0525</v>
       </c>
       <c r="H90" t="n">
-        <v>0.0771</v>
+        <v>0.0842</v>
       </c>
       <c r="I90" t="n">
         <v>90</v>
@@ -3712,10 +3712,10 @@
         <v>2.79</v>
       </c>
       <c r="G91" t="n">
-        <v>0.0483</v>
+        <v>0.0523</v>
       </c>
       <c r="H91" t="n">
-        <v>0.0759</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="I91" t="n">
         <v>88</v>
@@ -3748,10 +3748,10 @@
         <v>5.04</v>
       </c>
       <c r="G92" t="n">
-        <v>0.1119</v>
+        <v>0.0823</v>
       </c>
       <c r="H92" t="n">
-        <v>0.0974</v>
+        <v>0.0625</v>
       </c>
       <c r="I92" t="n">
         <v>89</v>
@@ -3784,10 +3784,10 @@
         <v>5.04</v>
       </c>
       <c r="G93" t="n">
-        <v>0.1127</v>
+        <v>0.0825</v>
       </c>
       <c r="H93" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="I93" t="n">
         <v>88</v>
@@ -3820,10 +3820,10 @@
         <v>5.04</v>
       </c>
       <c r="G94" t="n">
-        <v>0.105</v>
+        <v>0.081</v>
       </c>
       <c r="H94" t="n">
-        <v>0.0914</v>
+        <v>0.0613</v>
       </c>
       <c r="I94" t="n">
         <v>87</v>
@@ -3856,10 +3856,10 @@
         <v>6.49</v>
       </c>
       <c r="G95" t="n">
-        <v>0.0555</v>
+        <v>0.0669</v>
       </c>
       <c r="H95" t="n">
-        <v>0.0375</v>
+        <v>0.0462</v>
       </c>
       <c r="I95" t="n">
         <v>89</v>
@@ -3892,10 +3892,10 @@
         <v>6.49</v>
       </c>
       <c r="G96" t="n">
-        <v>0.0588</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="H96" t="n">
-        <v>0.0398</v>
+        <v>0.0467</v>
       </c>
       <c r="I96" t="n">
         <v>91</v>
@@ -3928,10 +3928,10 @@
         <v>6.49</v>
       </c>
       <c r="G97" t="n">
-        <v>0.0572</v>
+        <v>0.0673</v>
       </c>
       <c r="H97" t="n">
-        <v>0.0387</v>
+        <v>0.0464</v>
       </c>
       <c r="I97" t="n">
         <v>88</v>
@@ -3964,10 +3964,10 @@
         <v>4.29</v>
       </c>
       <c r="G98" t="n">
-        <v>0.0607</v>
+        <v>0.0696</v>
       </c>
       <c r="H98" t="n">
-        <v>0.0621</v>
+        <v>0.0726</v>
       </c>
       <c r="I98" t="n">
         <v>90</v>
@@ -4000,10 +4000,10 @@
         <v>4.29</v>
       </c>
       <c r="G99" t="n">
-        <v>0.061</v>
+        <v>0.0696</v>
       </c>
       <c r="H99" t="n">
-        <v>0.0624</v>
+        <v>0.0727</v>
       </c>
       <c r="I99" t="n">
         <v>91</v>
@@ -4036,10 +4036,10 @@
         <v>4.29</v>
       </c>
       <c r="G100" t="n">
-        <v>0.0633</v>
+        <v>0.0701</v>
       </c>
       <c r="H100" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0731</v>
       </c>
       <c r="I100" t="n">
         <v>91</v>
@@ -4072,10 +4072,10 @@
         <v>4.09</v>
       </c>
       <c r="G101" t="n">
-        <v>0.0569</v>
+        <v>0.0622</v>
       </c>
       <c r="H101" t="n">
-        <v>0.061</v>
+        <v>0.06809999999999999</v>
       </c>
       <c r="I101" t="n">
         <v>91</v>
@@ -4108,10 +4108,10 @@
         <v>4.09</v>
       </c>
       <c r="G102" t="n">
-        <v>0.0563</v>
+        <v>0.0621</v>
       </c>
       <c r="H102" t="n">
-        <v>0.0604</v>
+        <v>0.068</v>
       </c>
       <c r="I102" t="n">
         <v>91</v>
@@ -4144,10 +4144,10 @@
         <v>4.09</v>
       </c>
       <c r="G103" t="n">
-        <v>0.0579</v>
+        <v>0.0624</v>
       </c>
       <c r="H103" t="n">
-        <v>0.0621</v>
+        <v>0.0683</v>
       </c>
       <c r="I103" t="n">
         <v>91</v>
@@ -4180,10 +4180,10 @@
         <v>2.79</v>
       </c>
       <c r="G104" t="n">
-        <v>0.0479</v>
+        <v>0.0522</v>
       </c>
       <c r="H104" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0839</v>
       </c>
       <c r="I104" t="n">
         <v>88</v>
@@ -4216,10 +4216,10 @@
         <v>2.79</v>
       </c>
       <c r="G105" t="n">
-        <v>0.0471</v>
+        <v>0.0521</v>
       </c>
       <c r="H105" t="n">
-        <v>0.0741</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="I105" t="n">
         <v>90</v>
@@ -4252,10 +4252,10 @@
         <v>2.79</v>
       </c>
       <c r="G106" t="n">
-        <v>0.0478</v>
+        <v>0.0522</v>
       </c>
       <c r="H106" t="n">
-        <v>0.0752</v>
+        <v>0.0838</v>
       </c>
       <c r="I106" t="n">
         <v>90</v>
@@ -4288,10 +4288,10 @@
         <v>5.04</v>
       </c>
       <c r="G107" t="n">
-        <v>0.1079</v>
+        <v>0.0815</v>
       </c>
       <c r="H107" t="n">
-        <v>0.0936</v>
+        <v>0.0617</v>
       </c>
       <c r="I107" t="n">
         <v>93</v>
@@ -4324,10 +4324,10 @@
         <v>5.04</v>
       </c>
       <c r="G108" t="n">
-        <v>0.1061</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="H108" t="n">
-        <v>0.0921</v>
+        <v>0.0614</v>
       </c>
       <c r="I108" t="n">
         <v>93</v>
@@ -4360,10 +4360,10 @@
         <v>5.04</v>
       </c>
       <c r="G109" t="n">
-        <v>0.1077</v>
+        <v>0.0815</v>
       </c>
       <c r="H109" t="n">
-        <v>0.0935</v>
+        <v>0.0617</v>
       </c>
       <c r="I109" t="n">
         <v>93</v>
@@ -4396,10 +4396,10 @@
         <v>6.49</v>
       </c>
       <c r="G110" t="n">
-        <v>0.0572</v>
+        <v>0.0673</v>
       </c>
       <c r="H110" t="n">
-        <v>0.0386</v>
+        <v>0.0464</v>
       </c>
       <c r="I110" t="n">
         <v>90</v>
@@ -4432,10 +4432,10 @@
         <v>6.49</v>
       </c>
       <c r="G111" t="n">
-        <v>0.0571</v>
+        <v>0.0673</v>
       </c>
       <c r="H111" t="n">
-        <v>0.0384</v>
+        <v>0.0464</v>
       </c>
       <c r="I111" t="n">
         <v>88</v>
@@ -4468,10 +4468,10 @@
         <v>6.49</v>
       </c>
       <c r="G112" t="n">
-        <v>0.056</v>
+        <v>0.06710000000000001</v>
       </c>
       <c r="H112" t="n">
-        <v>0.0377</v>
+        <v>0.0463</v>
       </c>
       <c r="I112" t="n">
         <v>92</v>
@@ -4504,10 +4504,10 @@
         <v>4.29</v>
       </c>
       <c r="G113" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0703</v>
       </c>
       <c r="H113" t="n">
-        <v>0.0659</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="I113" t="n">
         <v>91</v>
@@ -4540,10 +4540,10 @@
         <v>4.29</v>
       </c>
       <c r="G114" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0704</v>
       </c>
       <c r="H114" t="n">
-        <v>0.0664</v>
+        <v>0.0735</v>
       </c>
       <c r="I114" t="n">
         <v>91</v>
@@ -4576,10 +4576,10 @@
         <v>4.29</v>
       </c>
       <c r="G115" t="n">
-        <v>0.0615</v>
+        <v>0.0697</v>
       </c>
       <c r="H115" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.0728</v>
       </c>
       <c r="I115" t="n">
         <v>90</v>
@@ -4612,10 +4612,10 @@
         <v>4.09</v>
       </c>
       <c r="G116" t="n">
-        <v>0.0583</v>
+        <v>0.0625</v>
       </c>
       <c r="H116" t="n">
-        <v>0.0623</v>
+        <v>0.0684</v>
       </c>
       <c r="I116" t="n">
         <v>90</v>
@@ -4648,10 +4648,10 @@
         <v>4.09</v>
       </c>
       <c r="G117" t="n">
-        <v>0.0542</v>
+        <v>0.0617</v>
       </c>
       <c r="H117" t="n">
-        <v>0.0579</v>
+        <v>0.0675</v>
       </c>
       <c r="I117" t="n">
         <v>88</v>
@@ -4684,10 +4684,10 @@
         <v>4.09</v>
       </c>
       <c r="G118" t="n">
-        <v>0.0583</v>
+        <v>0.0625</v>
       </c>
       <c r="H118" t="n">
-        <v>0.0623</v>
+        <v>0.0684</v>
       </c>
       <c r="I118" t="n">
         <v>91</v>
@@ -4720,10 +4720,10 @@
         <v>2.79</v>
       </c>
       <c r="G119" t="n">
-        <v>0.05</v>
+        <v>0.0527</v>
       </c>
       <c r="H119" t="n">
-        <v>0.0784</v>
+        <v>0.08450000000000001</v>
       </c>
       <c r="I119" t="n">
         <v>88</v>
@@ -4756,10 +4756,10 @@
         <v>2.79</v>
       </c>
       <c r="G120" t="n">
-        <v>0.0464</v>
+        <v>0.052</v>
       </c>
       <c r="H120" t="n">
-        <v>0.0727</v>
+        <v>0.0834</v>
       </c>
       <c r="I120" t="n">
         <v>91</v>
@@ -4792,10 +4792,10 @@
         <v>2.79</v>
       </c>
       <c r="G121" t="n">
-        <v>0.0493</v>
+        <v>0.0525</v>
       </c>
       <c r="H121" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.0843</v>
       </c>
       <c r="I121" t="n">
         <v>92</v>
@@ -4828,10 +4828,10 @@
         <v>6.29</v>
       </c>
       <c r="G122" t="n">
-        <v>0.0626</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="H122" t="n">
-        <v>0.0442</v>
+        <v>0.0521</v>
       </c>
       <c r="I122" t="n">
         <v>89</v>
@@ -4864,10 +4864,10 @@
         <v>6.29</v>
       </c>
       <c r="G123" t="n">
-        <v>0.06279999999999999</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="H123" t="n">
-        <v>0.0443</v>
+        <v>0.0521</v>
       </c>
       <c r="I123" t="n">
         <v>91</v>
@@ -4900,10 +4900,10 @@
         <v>6.29</v>
       </c>
       <c r="G124" t="n">
-        <v>0.0618</v>
+        <v>0.0728</v>
       </c>
       <c r="H124" t="n">
-        <v>0.0436</v>
+        <v>0.052</v>
       </c>
       <c r="I124" t="n">
         <v>92</v>
@@ -4936,10 +4936,10 @@
         <v>6.49</v>
       </c>
       <c r="G125" t="n">
-        <v>0.0755</v>
+        <v>0.0708</v>
       </c>
       <c r="H125" t="n">
-        <v>0.0517</v>
+        <v>0.049</v>
       </c>
       <c r="I125" t="n">
         <v>89</v>
@@ -4972,10 +4972,10 @@
         <v>6.49</v>
       </c>
       <c r="G126" t="n">
-        <v>0.0742</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="H126" t="n">
-        <v>0.0507</v>
+        <v>0.0488</v>
       </c>
       <c r="I126" t="n">
         <v>91</v>
@@ -5008,10 +5008,10 @@
         <v>6.49</v>
       </c>
       <c r="G127" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0701</v>
       </c>
       <c r="H127" t="n">
-        <v>0.0493</v>
+        <v>0.0485</v>
       </c>
       <c r="I127" t="n">
         <v>92</v>
@@ -5044,10 +5044,10 @@
         <v>4.29</v>
       </c>
       <c r="G128" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="H128" t="n">
-        <v>0.0755</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="I128" t="n">
         <v>88</v>
@@ -5080,10 +5080,10 @@
         <v>4.29</v>
       </c>
       <c r="G129" t="n">
-        <v>0.0732</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H129" t="n">
-        <v>0.0757</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="I129" t="n">
         <v>88</v>
@@ -5116,10 +5116,10 @@
         <v>4.29</v>
       </c>
       <c r="G130" t="n">
-        <v>0.0746</v>
+        <v>0.0722</v>
       </c>
       <c r="H130" t="n">
-        <v>0.0772</v>
+        <v>0.0756</v>
       </c>
       <c r="I130" t="n">
         <v>91</v>
@@ -5152,10 +5152,10 @@
         <v>4.09</v>
       </c>
       <c r="G131" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0644</v>
       </c>
       <c r="H131" t="n">
-        <v>0.0745</v>
+        <v>0.0707</v>
       </c>
       <c r="I131" t="n">
         <v>89</v>
@@ -5188,10 +5188,10 @@
         <v>4.09</v>
       </c>
       <c r="G132" t="n">
-        <v>0.0675</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="H132" t="n">
-        <v>0.0733</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="I132" t="n">
         <v>88</v>
@@ -5224,10 +5224,10 @@
         <v>4.09</v>
       </c>
       <c r="G133" t="n">
-        <v>0.0648</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="H133" t="n">
-        <v>0.0703</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I133" t="n">
         <v>90</v>
@@ -5260,10 +5260,10 @@
         <v>2.79</v>
       </c>
       <c r="G134" t="n">
-        <v>0.0572</v>
+        <v>0.054</v>
       </c>
       <c r="H134" t="n">
-        <v>0.0911</v>
+        <v>0.08690000000000001</v>
       </c>
       <c r="I134" t="n">
         <v>91</v>
@@ -5296,10 +5296,10 @@
         <v>2.79</v>
       </c>
       <c r="G135" t="n">
-        <v>0.0551</v>
+        <v>0.0536</v>
       </c>
       <c r="H135" t="n">
-        <v>0.0877</v>
+        <v>0.0863</v>
       </c>
       <c r="I135" t="n">
         <v>89</v>
@@ -5332,10 +5332,10 @@
         <v>2.79</v>
       </c>
       <c r="G136" t="n">
-        <v>0.0572</v>
+        <v>0.054</v>
       </c>
       <c r="H136" t="n">
-        <v>0.091</v>
+        <v>0.08690000000000001</v>
       </c>
       <c r="I136" t="n">
         <v>89</v>
@@ -5368,10 +5368,10 @@
         <v>6.29</v>
       </c>
       <c r="G137" t="n">
-        <v>0.066</v>
+        <v>0.0735</v>
       </c>
       <c r="H137" t="n">
-        <v>0.0469</v>
+        <v>0.0526</v>
       </c>
       <c r="I137" t="n">
         <v>90</v>
@@ -5404,10 +5404,10 @@
         <v>6.29</v>
       </c>
       <c r="G138" t="n">
-        <v>0.0643</v>
+        <v>0.0732</v>
       </c>
       <c r="H138" t="n">
-        <v>0.0457</v>
+        <v>0.0523</v>
       </c>
       <c r="I138" t="n">
         <v>90</v>
@@ -5440,10 +5440,10 @@
         <v>6.29</v>
       </c>
       <c r="G139" t="n">
-        <v>0.066</v>
+        <v>0.0735</v>
       </c>
       <c r="H139" t="n">
-        <v>0.0469</v>
+        <v>0.0526</v>
       </c>
       <c r="I139" t="n">
         <v>90</v>
@@ -5476,10 +5476,10 @@
         <v>6.49</v>
       </c>
       <c r="G140" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0702</v>
       </c>
       <c r="H140" t="n">
-        <v>0.0499</v>
+        <v>0.0487</v>
       </c>
       <c r="I140" t="n">
         <v>89</v>
@@ -5512,10 +5512,10 @@
         <v>6.49</v>
       </c>
       <c r="G141" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0707</v>
       </c>
       <c r="H141" t="n">
-        <v>0.0519</v>
+        <v>0.049</v>
       </c>
       <c r="I141" t="n">
         <v>88</v>
@@ -5548,10 +5548,10 @@
         <v>6.49</v>
       </c>
       <c r="G142" t="n">
-        <v>0.0736</v>
+        <v>0.0704</v>
       </c>
       <c r="H142" t="n">
-        <v>0.0507</v>
+        <v>0.0488</v>
       </c>
       <c r="I142" t="n">
         <v>91</v>
@@ -5584,10 +5584,10 @@
         <v>4.29</v>
       </c>
       <c r="G143" t="n">
-        <v>0.0725</v>
+        <v>0.0718</v>
       </c>
       <c r="H143" t="n">
-        <v>0.0756</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="I143" t="n">
         <v>89</v>
@@ -5620,10 +5620,10 @@
         <v>4.29</v>
       </c>
       <c r="G144" t="n">
-        <v>0.0771</v>
+        <v>0.0727</v>
       </c>
       <c r="H144" t="n">
-        <v>0.0804</v>
+        <v>0.0762</v>
       </c>
       <c r="I144" t="n">
         <v>91</v>
@@ -5656,10 +5656,10 @@
         <v>4.29</v>
       </c>
       <c r="G145" t="n">
-        <v>0.0747</v>
+        <v>0.0722</v>
       </c>
       <c r="H145" t="n">
-        <v>0.0779</v>
+        <v>0.0757</v>
       </c>
       <c r="I145" t="n">
         <v>88</v>
@@ -5692,10 +5692,10 @@
         <v>4.09</v>
       </c>
       <c r="G146" t="n">
-        <v>0.0643</v>
+        <v>0.0636</v>
       </c>
       <c r="H146" t="n">
-        <v>0.0703</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I146" t="n">
         <v>88</v>
@@ -5728,10 +5728,10 @@
         <v>4.09</v>
       </c>
       <c r="G147" t="n">
-        <v>0.0644</v>
+        <v>0.0636</v>
       </c>
       <c r="H147" t="n">
-        <v>0.0704</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I147" t="n">
         <v>89</v>
@@ -5764,10 +5764,10 @@
         <v>4.09</v>
       </c>
       <c r="G148" t="n">
-        <v>0.0672</v>
+        <v>0.0641</v>
       </c>
       <c r="H148" t="n">
-        <v>0.0735</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="I148" t="n">
         <v>90</v>
@@ -5800,10 +5800,10 @@
         <v>2.79</v>
       </c>
       <c r="G149" t="n">
-        <v>0.0536</v>
+        <v>0.0533</v>
       </c>
       <c r="H149" t="n">
-        <v>0.0859</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="I149" t="n">
         <v>89</v>
@@ -5836,10 +5836,10 @@
         <v>2.79</v>
       </c>
       <c r="G150" t="n">
-        <v>0.0546</v>
+        <v>0.0535</v>
       </c>
       <c r="H150" t="n">
-        <v>0.0876</v>
+        <v>0.0863</v>
       </c>
       <c r="I150" t="n">
         <v>91</v>
@@ -5872,10 +5872,10 @@
         <v>2.79</v>
       </c>
       <c r="G151" t="n">
-        <v>0.054</v>
+        <v>0.0534</v>
       </c>
       <c r="H151" t="n">
-        <v>0.08649999999999999</v>
+        <v>0.0861</v>
       </c>
       <c r="I151" t="n">
         <v>89</v>
@@ -5908,10 +5908,10 @@
         <v>6.29</v>
       </c>
       <c r="G152" t="n">
-        <v>0.06569999999999999</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="H152" t="n">
-        <v>0.0464</v>
+        <v>0.0525</v>
       </c>
       <c r="I152" t="n">
         <v>92</v>
@@ -5944,10 +5944,10 @@
         <v>6.29</v>
       </c>
       <c r="G153" t="n">
-        <v>0.066</v>
+        <v>0.0735</v>
       </c>
       <c r="H153" t="n">
-        <v>0.0467</v>
+        <v>0.0525</v>
       </c>
       <c r="I153" t="n">
         <v>92</v>
@@ -5980,10 +5980,10 @@
         <v>6.29</v>
       </c>
       <c r="G154" t="n">
-        <v>0.063</v>
+        <v>0.073</v>
       </c>
       <c r="H154" t="n">
-        <v>0.0446</v>
+        <v>0.0521</v>
       </c>
       <c r="I154" t="n">
         <v>88</v>
@@ -6016,10 +6016,10 @@
         <v>6.49</v>
       </c>
       <c r="G155" t="n">
-        <v>0.0725</v>
+        <v>0.0702</v>
       </c>
       <c r="H155" t="n">
-        <v>0.0497</v>
+        <v>0.0486</v>
       </c>
       <c r="I155" t="n">
         <v>90</v>
@@ -6052,10 +6052,10 @@
         <v>6.49</v>
       </c>
       <c r="G156" t="n">
-        <v>0.07149999999999999</v>
+        <v>0.0701</v>
       </c>
       <c r="H156" t="n">
-        <v>0.049</v>
+        <v>0.0485</v>
       </c>
       <c r="I156" t="n">
         <v>90</v>
@@ -6088,10 +6088,10 @@
         <v>6.49</v>
       </c>
       <c r="G157" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0701</v>
       </c>
       <c r="H157" t="n">
-        <v>0.0493</v>
+        <v>0.0486</v>
       </c>
       <c r="I157" t="n">
         <v>88</v>
@@ -6124,10 +6124,10 @@
         <v>4.29</v>
       </c>
       <c r="G158" t="n">
-        <v>0.0721</v>
+        <v>0.0718</v>
       </c>
       <c r="H158" t="n">
-        <v>0.0747</v>
+        <v>0.0752</v>
       </c>
       <c r="I158" t="n">
         <v>89</v>
@@ -6160,10 +6160,10 @@
         <v>4.29</v>
       </c>
       <c r="G159" t="n">
-        <v>0.0761</v>
+        <v>0.0725</v>
       </c>
       <c r="H159" t="n">
-        <v>0.079</v>
+        <v>0.0759</v>
       </c>
       <c r="I159" t="n">
         <v>92</v>
@@ -6196,10 +6196,10 @@
         <v>4.29</v>
       </c>
       <c r="G160" t="n">
-        <v>0.0771</v>
+        <v>0.0727</v>
       </c>
       <c r="H160" t="n">
-        <v>0.0799</v>
+        <v>0.0761</v>
       </c>
       <c r="I160" t="n">
         <v>88</v>
@@ -6232,10 +6232,10 @@
         <v>4.09</v>
       </c>
       <c r="G161" t="n">
-        <v>0.0634</v>
+        <v>0.0635</v>
       </c>
       <c r="H161" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.0697</v>
       </c>
       <c r="I161" t="n">
         <v>90</v>
@@ -6268,10 +6268,10 @@
         <v>4.09</v>
       </c>
       <c r="G162" t="n">
-        <v>0.0664</v>
+        <v>0.064</v>
       </c>
       <c r="H162" t="n">
-        <v>0.0723</v>
+        <v>0.0703</v>
       </c>
       <c r="I162" t="n">
         <v>92</v>
@@ -6304,10 +6304,10 @@
         <v>4.09</v>
       </c>
       <c r="G163" t="n">
-        <v>0.0673</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="H163" t="n">
-        <v>0.0732</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="I163" t="n">
         <v>89</v>
@@ -6340,10 +6340,10 @@
         <v>2.79</v>
       </c>
       <c r="G164" t="n">
-        <v>0.0544</v>
+        <v>0.0535</v>
       </c>
       <c r="H164" t="n">
-        <v>0.0867</v>
+        <v>0.0861</v>
       </c>
       <c r="I164" t="n">
         <v>90</v>
@@ -6376,10 +6376,10 @@
         <v>2.79</v>
       </c>
       <c r="G165" t="n">
-        <v>0.0566</v>
+        <v>0.0539</v>
       </c>
       <c r="H165" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.0868</v>
       </c>
       <c r="I165" t="n">
         <v>92</v>
@@ -6412,10 +6412,10 @@
         <v>2.79</v>
       </c>
       <c r="G166" t="n">
-        <v>0.0559</v>
+        <v>0.0538</v>
       </c>
       <c r="H166" t="n">
-        <v>0.0892</v>
+        <v>0.0866</v>
       </c>
       <c r="I166" t="n">
         <v>90</v>
@@ -6448,10 +6448,10 @@
         <v>6.29</v>
       </c>
       <c r="G167" t="n">
-        <v>0.0648</v>
+        <v>0.0733</v>
       </c>
       <c r="H167" t="n">
-        <v>0.0459</v>
+        <v>0.0524</v>
       </c>
       <c r="I167" t="n">
         <v>92</v>
@@ -6484,10 +6484,10 @@
         <v>6.29</v>
       </c>
       <c r="G168" t="n">
-        <v>0.0644</v>
+        <v>0.0732</v>
       </c>
       <c r="H168" t="n">
-        <v>0.0456</v>
+        <v>0.0523</v>
       </c>
       <c r="I168" t="n">
         <v>89</v>
@@ -6520,10 +6520,10 @@
         <v>6.29</v>
       </c>
       <c r="G169" t="n">
-        <v>0.0692</v>
+        <v>0.0741</v>
       </c>
       <c r="H169" t="n">
-        <v>0.049</v>
+        <v>0.0529</v>
       </c>
       <c r="I169" t="n">
         <v>90</v>
@@ -6556,10 +6556,10 @@
         <v>6.49</v>
       </c>
       <c r="G170" t="n">
-        <v>0.0708</v>
+        <v>0.0699</v>
       </c>
       <c r="H170" t="n">
-        <v>0.0486</v>
+        <v>0.0484</v>
       </c>
       <c r="I170" t="n">
         <v>92</v>
@@ -6592,10 +6592,10 @@
         <v>6.49</v>
       </c>
       <c r="G171" t="n">
-        <v>0.0722</v>
+        <v>0.0702</v>
       </c>
       <c r="H171" t="n">
-        <v>0.0495</v>
+        <v>0.0486</v>
       </c>
       <c r="I171" t="n">
         <v>88</v>
@@ -6628,10 +6628,10 @@
         <v>6.49</v>
       </c>
       <c r="G172" t="n">
-        <v>0.0698</v>
+        <v>0.0697</v>
       </c>
       <c r="H172" t="n">
-        <v>0.0479</v>
+        <v>0.0483</v>
       </c>
       <c r="I172" t="n">
         <v>89</v>
@@ -6664,10 +6664,10 @@
         <v>4.29</v>
       </c>
       <c r="G173" t="n">
-        <v>0.0737</v>
+        <v>0.0721</v>
       </c>
       <c r="H173" t="n">
-        <v>0.0765</v>
+        <v>0.0755</v>
       </c>
       <c r="I173" t="n">
         <v>88</v>
@@ -6700,10 +6700,10 @@
         <v>4.29</v>
       </c>
       <c r="G174" t="n">
-        <v>0.0767</v>
+        <v>0.0726</v>
       </c>
       <c r="H174" t="n">
-        <v>0.0796</v>
+        <v>0.076</v>
       </c>
       <c r="I174" t="n">
         <v>89</v>
@@ -6736,10 +6736,10 @@
         <v>4.29</v>
       </c>
       <c r="G175" t="n">
-        <v>0.0742</v>
+        <v>0.0722</v>
       </c>
       <c r="H175" t="n">
-        <v>0.077</v>
+        <v>0.0756</v>
       </c>
       <c r="I175" t="n">
         <v>89</v>
@@ -6772,10 +6772,10 @@
         <v>4.09</v>
       </c>
       <c r="G176" t="n">
-        <v>0.0682</v>
+        <v>0.0643</v>
       </c>
       <c r="H176" t="n">
-        <v>0.0742</v>
+        <v>0.0707</v>
       </c>
       <c r="I176" t="n">
         <v>91</v>
@@ -6808,10 +6808,10 @@
         <v>4.09</v>
       </c>
       <c r="G177" t="n">
-        <v>0.0644</v>
+        <v>0.0636</v>
       </c>
       <c r="H177" t="n">
-        <v>0.0701</v>
+        <v>0.0699</v>
       </c>
       <c r="I177" t="n">
         <v>88</v>
@@ -6844,10 +6844,10 @@
         <v>4.09</v>
       </c>
       <c r="G178" t="n">
-        <v>0.06569999999999999</v>
+        <v>0.0639</v>
       </c>
       <c r="H178" t="n">
-        <v>0.07149999999999999</v>
+        <v>0.0702</v>
       </c>
       <c r="I178" t="n">
         <v>91</v>
@@ -6880,10 +6880,10 @@
         <v>2.79</v>
       </c>
       <c r="G179" t="n">
-        <v>0.0567</v>
+        <v>0.0539</v>
       </c>
       <c r="H179" t="n">
-        <v>0.0905</v>
+        <v>0.0868</v>
       </c>
       <c r="I179" t="n">
         <v>89</v>
@@ -6916,10 +6916,10 @@
         <v>2.79</v>
       </c>
       <c r="G180" t="n">
-        <v>0.0549</v>
+        <v>0.0536</v>
       </c>
       <c r="H180" t="n">
-        <v>0.0876</v>
+        <v>0.0863</v>
       </c>
       <c r="I180" t="n">
         <v>89</v>
@@ -6952,10 +6952,10 @@
         <v>2.79</v>
       </c>
       <c r="G181" t="n">
-        <v>0.0542</v>
+        <v>0.0535</v>
       </c>
       <c r="H181" t="n">
-        <v>0.0864</v>
+        <v>0.0861</v>
       </c>
       <c r="I181" t="n">
         <v>89</v>
@@ -6988,10 +6988,10 @@
         <v>6.29</v>
       </c>
       <c r="G182" t="n">
-        <v>0.07049999999999999</v>
+        <v>0.0762</v>
       </c>
       <c r="H182" t="n">
-        <v>0.0502</v>
+        <v>0.0546</v>
       </c>
       <c r="I182" t="n">
         <v>92</v>
@@ -7024,10 +7024,10 @@
         <v>6.29</v>
       </c>
       <c r="G183" t="n">
-        <v>0.0692</v>
+        <v>0.0759</v>
       </c>
       <c r="H183" t="n">
-        <v>0.0492</v>
+        <v>0.0544</v>
       </c>
       <c r="I183" t="n">
         <v>91</v>
@@ -7060,10 +7060,10 @@
         <v>6.29</v>
       </c>
       <c r="G184" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="H184" t="n">
-        <v>0.0488</v>
+        <v>0.0543</v>
       </c>
       <c r="I184" t="n">
         <v>91</v>
@@ -7096,10 +7096,10 @@
         <v>6.49</v>
       </c>
       <c r="G185" t="n">
-        <v>0.0736</v>
+        <v>0.0699</v>
       </c>
       <c r="H185" t="n">
-        <v>0.0507</v>
+        <v>0.0485</v>
       </c>
       <c r="I185" t="n">
         <v>91</v>
@@ -7132,10 +7132,10 @@
         <v>6.49</v>
       </c>
       <c r="G186" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0696</v>
       </c>
       <c r="H186" t="n">
-        <v>0.0496</v>
+        <v>0.0484</v>
       </c>
       <c r="I186" t="n">
         <v>92</v>
@@ -7168,10 +7168,10 @@
         <v>6.49</v>
       </c>
       <c r="G187" t="n">
-        <v>0.0699</v>
+        <v>0.0693</v>
       </c>
       <c r="H187" t="n">
-        <v>0.0482</v>
+        <v>0.0481</v>
       </c>
       <c r="I187" t="n">
         <v>89</v>
@@ -7204,10 +7204,10 @@
         <v>4.29</v>
       </c>
       <c r="G188" t="n">
-        <v>0.0759</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="H188" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.0756</v>
       </c>
       <c r="I188" t="n">
         <v>88</v>
@@ -7240,10 +7240,10 @@
         <v>4.29</v>
       </c>
       <c r="G189" t="n">
-        <v>0.0726</v>
+        <v>0.0713</v>
       </c>
       <c r="H189" t="n">
-        <v>0.07580000000000001</v>
+        <v>0.075</v>
       </c>
       <c r="I189" t="n">
         <v>90</v>
@@ -7276,10 +7276,10 @@
         <v>4.29</v>
       </c>
       <c r="G190" t="n">
-        <v>0.0709</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H190" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.0746</v>
       </c>
       <c r="I190" t="n">
         <v>90</v>
@@ -7312,10 +7312,10 @@
         <v>4.09</v>
       </c>
       <c r="G191" t="n">
-        <v>0.06510000000000001</v>
+        <v>0.0633</v>
       </c>
       <c r="H191" t="n">
-        <v>0.0712</v>
+        <v>0.0698</v>
       </c>
       <c r="I191" t="n">
         <v>88</v>
@@ -7348,10 +7348,10 @@
         <v>4.09</v>
       </c>
       <c r="G192" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.063</v>
       </c>
       <c r="H192" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.0694</v>
       </c>
       <c r="I192" t="n">
         <v>91</v>
@@ -7384,10 +7384,10 @@
         <v>4.09</v>
       </c>
       <c r="G193" t="n">
-        <v>0.0638</v>
+        <v>0.0631</v>
       </c>
       <c r="H193" t="n">
-        <v>0.0698</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="I193" t="n">
         <v>88</v>
@@ -7420,10 +7420,10 @@
         <v>2.79</v>
       </c>
       <c r="G194" t="n">
-        <v>0.0558</v>
+        <v>0.0533</v>
       </c>
       <c r="H194" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.0862</v>
       </c>
       <c r="I194" t="n">
         <v>92</v>
@@ -7456,10 +7456,10 @@
         <v>2.79</v>
       </c>
       <c r="G195" t="n">
-        <v>0.0531</v>
+        <v>0.0529</v>
       </c>
       <c r="H195" t="n">
-        <v>0.0851</v>
+        <v>0.0854</v>
       </c>
       <c r="I195" t="n">
         <v>89</v>
@@ -7492,10 +7492,10 @@
         <v>2.79</v>
       </c>
       <c r="G196" t="n">
-        <v>0.056</v>
+        <v>0.0534</v>
       </c>
       <c r="H196" t="n">
-        <v>0.0898</v>
+        <v>0.0862</v>
       </c>
       <c r="I196" t="n">
         <v>88</v>
@@ -7528,10 +7528,10 @@
         <v>6.29</v>
       </c>
       <c r="G197" t="n">
-        <v>0.0699</v>
+        <v>0.0761</v>
       </c>
       <c r="H197" t="n">
-        <v>0.0496</v>
+        <v>0.0545</v>
       </c>
       <c r="I197" t="n">
         <v>92</v>
@@ -7564,10 +7564,10 @@
         <v>6.29</v>
       </c>
       <c r="G198" t="n">
-        <v>0.0707</v>
+        <v>0.0762</v>
       </c>
       <c r="H198" t="n">
-        <v>0.0502</v>
+        <v>0.0546</v>
       </c>
       <c r="I198" t="n">
         <v>90</v>
@@ -7600,10 +7600,10 @@
         <v>6.29</v>
       </c>
       <c r="G199" t="n">
-        <v>0.0708</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="H199" t="n">
-        <v>0.0503</v>
+        <v>0.0546</v>
       </c>
       <c r="I199" t="n">
         <v>90</v>
@@ -7636,10 +7636,10 @@
         <v>6.49</v>
       </c>
       <c r="G200" t="n">
-        <v>0.0693</v>
+        <v>0.0692</v>
       </c>
       <c r="H200" t="n">
-        <v>0.0477</v>
+        <v>0.048</v>
       </c>
       <c r="I200" t="n">
         <v>89</v>
@@ -7672,10 +7672,10 @@
         <v>6.49</v>
       </c>
       <c r="G201" t="n">
-        <v>0.0708</v>
+        <v>0.0694</v>
       </c>
       <c r="H201" t="n">
-        <v>0.0487</v>
+        <v>0.0482</v>
       </c>
       <c r="I201" t="n">
         <v>91</v>
@@ -7708,10 +7708,10 @@
         <v>6.49</v>
       </c>
       <c r="G202" t="n">
-        <v>0.0703</v>
+        <v>0.0693</v>
       </c>
       <c r="H202" t="n">
-        <v>0.0484</v>
+        <v>0.0481</v>
       </c>
       <c r="I202" t="n">
         <v>91</v>
@@ -7744,10 +7744,10 @@
         <v>4.29</v>
       </c>
       <c r="G203" t="n">
-        <v>0.07340000000000001</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="H203" t="n">
-        <v>0.0764</v>
+        <v>0.0751</v>
       </c>
       <c r="I203" t="n">
         <v>92</v>
@@ -7780,10 +7780,10 @@
         <v>4.29</v>
       </c>
       <c r="G204" t="n">
-        <v>0.07340000000000001</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="H204" t="n">
-        <v>0.0764</v>
+        <v>0.0751</v>
       </c>
       <c r="I204" t="n">
         <v>92</v>
@@ -7816,10 +7816,10 @@
         <v>4.29</v>
       </c>
       <c r="G205" t="n">
-        <v>0.0731</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="H205" t="n">
-        <v>0.0761</v>
+        <v>0.075</v>
       </c>
       <c r="I205" t="n">
         <v>90</v>
@@ -7852,10 +7852,10 @@
         <v>4.09</v>
       </c>
       <c r="G206" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="H206" t="n">
-        <v>0.0706</v>
+        <v>0.0697</v>
       </c>
       <c r="I206" t="n">
         <v>91</v>
@@ -7888,10 +7888,10 @@
         <v>4.09</v>
       </c>
       <c r="G207" t="n">
-        <v>0.0634</v>
+        <v>0.063</v>
       </c>
       <c r="H207" t="n">
-        <v>0.0693</v>
+        <v>0.0694</v>
       </c>
       <c r="I207" t="n">
         <v>91</v>
@@ -7924,10 +7924,10 @@
         <v>4.09</v>
       </c>
       <c r="G208" t="n">
-        <v>0.0631</v>
+        <v>0.0629</v>
       </c>
       <c r="H208" t="n">
-        <v>0.0689</v>
+        <v>0.0693</v>
       </c>
       <c r="I208" t="n">
         <v>89</v>
@@ -7960,10 +7960,10 @@
         <v>2.79</v>
       </c>
       <c r="G209" t="n">
-        <v>0.0537</v>
+        <v>0.053</v>
       </c>
       <c r="H209" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0856</v>
       </c>
       <c r="I209" t="n">
         <v>92</v>
@@ -7996,10 +7996,10 @@
         <v>2.79</v>
       </c>
       <c r="G210" t="n">
-        <v>0.0562</v>
+        <v>0.0534</v>
       </c>
       <c r="H210" t="n">
-        <v>0.08989999999999999</v>
+        <v>0.0863</v>
       </c>
       <c r="I210" t="n">
         <v>88</v>
@@ -8032,10 +8032,10 @@
         <v>2.79</v>
       </c>
       <c r="G211" t="n">
-        <v>0.0572</v>
+        <v>0.0536</v>
       </c>
       <c r="H211" t="n">
-        <v>0.0916</v>
+        <v>0.0866</v>
       </c>
       <c r="I211" t="n">
         <v>92</v>
@@ -8068,10 +8068,10 @@
         <v>6.29</v>
       </c>
       <c r="G212" t="n">
-        <v>0.0741</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="H212" t="n">
-        <v>0.0529</v>
+        <v>0.0551</v>
       </c>
       <c r="I212" t="n">
         <v>90</v>
@@ -8104,10 +8104,10 @@
         <v>6.29</v>
       </c>
       <c r="G213" t="n">
-        <v>0.0701</v>
+        <v>0.0761</v>
       </c>
       <c r="H213" t="n">
-        <v>0.0501</v>
+        <v>0.0546</v>
       </c>
       <c r="I213" t="n">
         <v>92</v>
@@ -8140,10 +8140,10 @@
         <v>6.29</v>
       </c>
       <c r="G214" t="n">
-        <v>0.07340000000000001</v>
+        <v>0.0767</v>
       </c>
       <c r="H214" t="n">
-        <v>0.0525</v>
+        <v>0.055</v>
       </c>
       <c r="I214" t="n">
         <v>89</v>
@@ -8176,10 +8176,10 @@
         <v>6.49</v>
       </c>
       <c r="G215" t="n">
-        <v>0.0682</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H215" t="n">
-        <v>0.0473</v>
+        <v>0.0479</v>
       </c>
       <c r="I215" t="n">
         <v>92</v>
@@ -8212,10 +8212,10 @@
         <v>6.49</v>
       </c>
       <c r="G216" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0697</v>
       </c>
       <c r="H216" t="n">
-        <v>0.0501</v>
+        <v>0.0484</v>
       </c>
       <c r="I216" t="n">
         <v>90</v>
@@ -8248,10 +8248,10 @@
         <v>6.49</v>
       </c>
       <c r="G217" t="n">
-        <v>0.0726</v>
+        <v>0.0697</v>
       </c>
       <c r="H217" t="n">
-        <v>0.0503</v>
+        <v>0.0485</v>
       </c>
       <c r="I217" t="n">
         <v>89</v>
@@ -8284,10 +8284,10 @@
         <v>4.29</v>
       </c>
       <c r="G218" t="n">
-        <v>0.0735</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="H218" t="n">
-        <v>0.077</v>
+        <v>0.0752</v>
       </c>
       <c r="I218" t="n">
         <v>90</v>
@@ -8320,10 +8320,10 @@
         <v>4.29</v>
       </c>
       <c r="G219" t="n">
-        <v>0.07489999999999999</v>
+        <v>0.0718</v>
       </c>
       <c r="H219" t="n">
-        <v>0.0785</v>
+        <v>0.0755</v>
       </c>
       <c r="I219" t="n">
         <v>90</v>
@@ -8356,10 +8356,10 @@
         <v>4.29</v>
       </c>
       <c r="G220" t="n">
-        <v>0.07049999999999999</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H220" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.0746</v>
       </c>
       <c r="I220" t="n">
         <v>89</v>
@@ -8392,10 +8392,10 @@
         <v>4.09</v>
       </c>
       <c r="G221" t="n">
-        <v>0.0633</v>
+        <v>0.063</v>
       </c>
       <c r="H221" t="n">
-        <v>0.0696</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="I221" t="n">
         <v>90</v>
@@ -8428,10 +8428,10 @@
         <v>4.09</v>
       </c>
       <c r="G222" t="n">
-        <v>0.0641</v>
+        <v>0.0631</v>
       </c>
       <c r="H222" t="n">
-        <v>0.0704</v>
+        <v>0.0696</v>
       </c>
       <c r="I222" t="n">
         <v>88</v>
@@ -8464,10 +8464,10 @@
         <v>4.09</v>
       </c>
       <c r="G223" t="n">
-        <v>0.0621</v>
+        <v>0.06279999999999999</v>
       </c>
       <c r="H223" t="n">
-        <v>0.0683</v>
+        <v>0.0692</v>
       </c>
       <c r="I223" t="n">
         <v>89</v>
@@ -8500,10 +8500,10 @@
         <v>2.79</v>
       </c>
       <c r="G224" t="n">
-        <v>0.0539</v>
+        <v>0.053</v>
       </c>
       <c r="H224" t="n">
-        <v>0.08690000000000001</v>
+        <v>0.0857</v>
       </c>
       <c r="I224" t="n">
         <v>90</v>
@@ -8536,10 +8536,10 @@
         <v>2.79</v>
       </c>
       <c r="G225" t="n">
-        <v>0.0531</v>
+        <v>0.0529</v>
       </c>
       <c r="H225" t="n">
-        <v>0.0856</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="I225" t="n">
         <v>90</v>
@@ -8572,10 +8572,10 @@
         <v>2.79</v>
       </c>
       <c r="G226" t="n">
-        <v>0.0537</v>
+        <v>0.053</v>
       </c>
       <c r="H226" t="n">
-        <v>0.08649999999999999</v>
+        <v>0.0857</v>
       </c>
       <c r="I226" t="n">
         <v>92</v>
@@ -8608,10 +8608,10 @@
         <v>6.29</v>
       </c>
       <c r="G227" t="n">
-        <v>0.0732</v>
+        <v>0.0766</v>
       </c>
       <c r="H227" t="n">
-        <v>0.0525</v>
+        <v>0.055</v>
       </c>
       <c r="I227" t="n">
         <v>88</v>
@@ -8680,10 +8680,10 @@
         <v>6.29</v>
       </c>
       <c r="G229" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.0772</v>
       </c>
       <c r="H229" t="n">
-        <v>0.0547</v>
+        <v>0.0554</v>
       </c>
       <c r="I229" t="n">
         <v>92</v>
@@ -8716,10 +8716,10 @@
         <v>6.49</v>
       </c>
       <c r="G230" t="n">
-        <v>0.07190000000000001</v>
+        <v>0.0696</v>
       </c>
       <c r="H230" t="n">
-        <v>0.05</v>
+        <v>0.0484</v>
       </c>
       <c r="I230" t="n">
         <v>88</v>
@@ -8752,10 +8752,10 @@
         <v>6.49</v>
       </c>
       <c r="G231" t="n">
-        <v>0.0712</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H231" t="n">
-        <v>0.0495</v>
+        <v>0.0483</v>
       </c>
       <c r="I231" t="n">
         <v>90</v>
@@ -8788,10 +8788,10 @@
         <v>6.49</v>
       </c>
       <c r="G232" t="n">
-        <v>0.0673</v>
+        <v>0.0688</v>
       </c>
       <c r="H232" t="n">
-        <v>0.0468</v>
+        <v>0.0478</v>
       </c>
       <c r="I232" t="n">
         <v>89</v>
@@ -8824,10 +8824,10 @@
         <v>4.29</v>
       </c>
       <c r="G233" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.0711</v>
       </c>
       <c r="H233" t="n">
-        <v>0.0751</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="I233" t="n">
         <v>91</v>
@@ -8860,10 +8860,10 @@
         <v>4.29</v>
       </c>
       <c r="G234" t="n">
-        <v>0.0694</v>
+        <v>0.0708</v>
       </c>
       <c r="H234" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="I234" t="n">
         <v>88</v>
@@ -8896,10 +8896,10 @@
         <v>4.29</v>
       </c>
       <c r="G235" t="n">
-        <v>0.0731</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="H235" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.0752</v>
       </c>
       <c r="I235" t="n">
         <v>92</v>
@@ -8932,10 +8932,10 @@
         <v>4.09</v>
       </c>
       <c r="G236" t="n">
-        <v>0.0635</v>
+        <v>0.063</v>
       </c>
       <c r="H236" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="I236" t="n">
         <v>92</v>
@@ -8968,10 +8968,10 @@
         <v>4.09</v>
       </c>
       <c r="G237" t="n">
-        <v>0.0619</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="H237" t="n">
-        <v>0.0682</v>
+        <v>0.0692</v>
       </c>
       <c r="I237" t="n">
         <v>88</v>
@@ -9004,10 +9004,10 @@
         <v>4.09</v>
       </c>
       <c r="G238" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0633</v>
       </c>
       <c r="H238" t="n">
-        <v>0.07190000000000001</v>
+        <v>0.0699</v>
       </c>
       <c r="I238" t="n">
         <v>89</v>
@@ -9040,10 +9040,10 @@
         <v>2.79</v>
       </c>
       <c r="G239" t="n">
-        <v>0.0513</v>
+        <v>0.0525</v>
       </c>
       <c r="H239" t="n">
-        <v>0.083</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="I239" t="n">
         <v>90</v>
@@ -9076,10 +9076,10 @@
         <v>2.79</v>
       </c>
       <c r="G240" t="n">
-        <v>0.0532</v>
+        <v>0.0529</v>
       </c>
       <c r="H240" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0856</v>
       </c>
       <c r="I240" t="n">
         <v>91</v>
@@ -9112,10 +9112,10 @@
         <v>2.79</v>
       </c>
       <c r="G241" t="n">
-        <v>0.0539</v>
+        <v>0.053</v>
       </c>
       <c r="H241" t="n">
-        <v>0.0871</v>
+        <v>0.0858</v>
       </c>
       <c r="I241" t="n">
         <v>90</v>

</xml_diff>